<commit_message>
Refresh Track aggregators automatically in daily pipeline
</commit_message>
<xml_diff>
--- a/backend/data/cargos_recurrentes/cargos_recurrentes.xlsx
+++ b/backend/data/cargos_recurrentes/cargos_recurrentes.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="234">
   <si>
     <t>Reporte Cargos Recurrentes</t>
   </si>
@@ -67,7 +67,7 @@
     <t>Unnamed: 16</t>
   </si>
   <si>
-    <t>Reporte generado: 01-05-2026 06:56 p. m.</t>
+    <t>Reporte generado: 02-05-2026 03:43 p. m.</t>
   </si>
   <si>
     <t>Folio</t>
@@ -79,6 +79,18 @@
     <t>PIN</t>
   </si>
   <si>
+    <t>02210</t>
+  </si>
+  <si>
+    <t>02967</t>
+  </si>
+  <si>
+    <t>03168</t>
+  </si>
+  <si>
+    <t>09964</t>
+  </si>
+  <si>
     <t>03052</t>
   </si>
   <si>
@@ -91,57 +103,87 @@
     <t>02922</t>
   </si>
   <si>
+    <t>02795</t>
+  </si>
+  <si>
     <t>03156</t>
   </si>
   <si>
+    <t>02589</t>
+  </si>
+  <si>
+    <t>03053</t>
+  </si>
+  <si>
+    <t>03183</t>
+  </si>
+  <si>
     <t>03034</t>
   </si>
   <si>
-    <t>02210</t>
-  </si>
-  <si>
-    <t>02967</t>
-  </si>
-  <si>
-    <t>03168</t>
+    <t>03191</t>
+  </si>
+  <si>
+    <t>03219</t>
   </si>
   <si>
     <t>09543</t>
   </si>
   <si>
-    <t>02589</t>
-  </si>
-  <si>
-    <t>03053</t>
-  </si>
-  <si>
     <t>03005</t>
   </si>
   <si>
     <t>03017</t>
   </si>
   <si>
+    <t>03221</t>
+  </si>
+  <si>
     <t>Nombre</t>
   </si>
   <si>
+    <t>BALTAZAR VILLASEÑOR  CRUZ</t>
+  </si>
+  <si>
+    <t>CESAR OMAR OBREGON ESTRELLLO</t>
+  </si>
+  <si>
+    <t>ANTONIO  LAMAS IRINEO</t>
+  </si>
+  <si>
+    <t>DEMIAN CORONADO LOPEZ</t>
+  </si>
+  <si>
+    <t>FELIPE ALFONSO GUERRERO INZUNZA</t>
+  </si>
+  <si>
+    <t>LILIAN RUVALCABA FIGUEROA</t>
+  </si>
+  <si>
+    <t>GUADALUPE  CASTRO ROSAS</t>
+  </si>
+  <si>
+    <t>MARIA DEL CARMEN JIMENEZ SANCHEZ</t>
+  </si>
+  <si>
+    <t>ZARAKY RENE  ZENTENO  ORTIZ</t>
+  </si>
+  <si>
+    <t>CARLA DANIELA MARTINEZ  GUILLEN</t>
+  </si>
+  <si>
+    <t>CARLOS EDUARDO  FLORES  SANCHEZ</t>
+  </si>
+  <si>
+    <t>MINERVA  GONZALEZ  MACEDO</t>
+  </si>
+  <si>
+    <t>EDUARDO  GONZALES FLORES</t>
+  </si>
+  <si>
     <t>LARISSA DENISSE LOPEZ BURGOS</t>
   </si>
   <si>
-    <t>MARIA DEL CARMEN JIMENEZ SANCHEZ</t>
-  </si>
-  <si>
-    <t>ZARAKY RENE  ZENTENO  ORTIZ</t>
-  </si>
-  <si>
-    <t>CARLA DANIELA MARTINEZ  GUILLEN</t>
-  </si>
-  <si>
-    <t>CARLOS EDUARDO  FLORES  SANCHEZ</t>
-  </si>
-  <si>
-    <t>MINERVA  GONZALEZ  MACEDO</t>
-  </si>
-  <si>
     <t>JOSE MANUEL OSUNA PEÑA</t>
   </si>
   <si>
@@ -151,9 +193,42 @@
     <t>MARLENE  GARCIA AGUILAR</t>
   </si>
   <si>
+    <t>NATALIA PADILLA RIVAS</t>
+  </si>
+  <si>
     <t>CESAR DANIEL  PEREYRA  CONTRERAS</t>
   </si>
   <si>
+    <t>ERIKA ADRIANA BERMUDEZ TALAVERA</t>
+  </si>
+  <si>
+    <t>ISRAEL CRESPO RIOS</t>
+  </si>
+  <si>
+    <t>JULIO CESAR VERDE  MANJARRES</t>
+  </si>
+  <si>
+    <t>JESUS ANTONIO ABRIL CAMPOS</t>
+  </si>
+  <si>
+    <t>MARA FERNANDA LUNA MENDOZA</t>
+  </si>
+  <si>
+    <t>NOEMI  RAMOS  DE LEON</t>
+  </si>
+  <si>
+    <t>DENIS LILIANA AMEZCUA CRUZ</t>
+  </si>
+  <si>
+    <t>LUIS DAVID ROSAS  ALONSO</t>
+  </si>
+  <si>
+    <t>ALMA ANGELICA  PEREZ  MIRANDA</t>
+  </si>
+  <si>
+    <t>ANGELICA DEYANIRA SERRANO VALDEZ</t>
+  </si>
+  <si>
     <t>ELISA ELENA PAREDES HERNANDEZ</t>
   </si>
   <si>
@@ -166,19 +241,49 @@
     <t>JOANNA VILLEGAS ORTIZ</t>
   </si>
   <si>
+    <t>JESUS ABELARDO RODRIGUEZ NAVARRO</t>
+  </si>
+  <si>
+    <t>HILARY MONROY MORENO</t>
+  </si>
+  <si>
     <t>MONICA DANIELA  ORDUÑO PEREZ</t>
   </si>
   <si>
-    <t>BALTAZAR VILLASEÑOR  CRUZ</t>
-  </si>
-  <si>
-    <t>CESAR OMAR OBREGON ESTRELLLO</t>
-  </si>
-  <si>
-    <t>ANTONIO  LAMAS IRINEO</t>
-  </si>
-  <si>
-    <t>DEMIAN CORONADO LOPEZ</t>
+    <t>JUAN JOSE  PACHECO  FLORES</t>
+  </si>
+  <si>
+    <t>DULCE NOHEMI SOTO MORENO</t>
+  </si>
+  <si>
+    <t>SUSAN ELIZABETH SOTO PIÑA</t>
+  </si>
+  <si>
+    <t>CHRISTIAN PRISCILA CARDONA BANDA</t>
+  </si>
+  <si>
+    <t>ALAN IGNACIO  CORTES HERNANDEZ</t>
+  </si>
+  <si>
+    <t>YOSHIO JESUS  RINCON  MIRANDA</t>
+  </si>
+  <si>
+    <t>LETICIA RUBIO VALENZUELA</t>
+  </si>
+  <si>
+    <t>BRISEIDA ISABEL ENRIQUEZ ZEPEDA</t>
+  </si>
+  <si>
+    <t>ANA LUISA  HERNANDEZ  BELTRAN</t>
+  </si>
+  <si>
+    <t>ANA FABIOLA FLORES CARMONA</t>
+  </si>
+  <si>
+    <t>GUILLERMO GERARDO VAZQUEZ GARCIA</t>
+  </si>
+  <si>
+    <t>JUAN  FLORES  FELIX</t>
   </si>
   <si>
     <t>ALEJANDRO MAGALLAN  LOPEZ</t>
@@ -187,40 +292,7 @@
     <t>NIRVANA FERNANDA  SALADO  SANCHEZ</t>
   </si>
   <si>
-    <t>ANA LUISA  HERNANDEZ  BELTRAN</t>
-  </si>
-  <si>
-    <t>ANA FABIOLA FLORES CARMONA</t>
-  </si>
-  <si>
-    <t>GUILLERMO GERARDO VAZQUEZ GARCIA</t>
-  </si>
-  <si>
-    <t>JUAN JOSE  PACHECO  FLORES</t>
-  </si>
-  <si>
-    <t>CHRISTIAN PRISCILA CARDONA BANDA</t>
-  </si>
-  <si>
-    <t>SUSAN ELIZABETH SOTO PIÑA</t>
-  </si>
-  <si>
-    <t>BRISEIDA ISABEL ENRIQUEZ ZEPEDA</t>
-  </si>
-  <si>
-    <t>ISRAEL CRESPO RIOS</t>
-  </si>
-  <si>
-    <t>MARA FERNANDA LUNA MENDOZA</t>
-  </si>
-  <si>
-    <t>NOEMI  RAMOS  DE LEON</t>
-  </si>
-  <si>
-    <t>JESUS ANTONIO ABRIL CAMPOS</t>
-  </si>
-  <si>
-    <t>ALMA ANGELICA  PEREZ  MIRANDA</t>
+    <t>ELOINA  REYNOSO  TERRONES</t>
   </si>
   <si>
     <t>TANIA ELIZABETH VILLAREAL PEREDA</t>
@@ -229,6 +301,9 @@
     <t>ELIUD RAMIREZ BELMARES</t>
   </si>
   <si>
+    <t>GILBERTO  BARRIOS HERNANDEZ</t>
+  </si>
+  <si>
     <t>JUAN FRANCISCO PITONES NORIEGA</t>
   </si>
   <si>
@@ -238,52 +313,58 @@
     <t>Sucursal</t>
   </si>
   <si>
+    <t>METEPEC</t>
+  </si>
+  <si>
+    <t>SALTILLO VILLALTA</t>
+  </si>
+  <si>
+    <t>SEND MXL</t>
+  </si>
+  <si>
     <t>TEC MXL</t>
   </si>
   <si>
+    <t>SEND CUL</t>
+  </si>
+  <si>
+    <t>MISION ENS</t>
+  </si>
+  <si>
     <t>SEND SALTILLO</t>
   </si>
   <si>
     <t>IXTAPALUCA</t>
   </si>
   <si>
-    <t>SEND MXL</t>
-  </si>
-  <si>
-    <t>METEPEC</t>
-  </si>
-  <si>
     <t>PASEO 2000</t>
   </si>
   <si>
     <t>VILLA VERDE</t>
   </si>
   <si>
-    <t>MISION ENS</t>
-  </si>
-  <si>
-    <t>SEND CUL</t>
-  </si>
-  <si>
-    <t>SALTILLO VILLALTA</t>
+    <t>CARROUSEL TJ</t>
+  </si>
+  <si>
+    <t>SAN LUIS</t>
+  </si>
+  <si>
+    <t>SANTA FE</t>
+  </si>
+  <si>
+    <t>STA CATARINA</t>
+  </si>
+  <si>
+    <t>INDEPENDENCIA</t>
+  </si>
+  <si>
+    <t>PAPALOTE TJ</t>
   </si>
   <si>
     <t>AZAHARES CUL</t>
   </si>
   <si>
-    <t>CARROUSEL TJ</t>
-  </si>
-  <si>
-    <t>STA CATARINA</t>
-  </si>
-  <si>
-    <t>PAPALOTE TJ</t>
-  </si>
-  <si>
-    <t>SAN LUIS</t>
-  </si>
-  <si>
-    <t>SANTA FE</t>
+    <t>PABELLON RTO</t>
   </si>
   <si>
     <t>INSURGENTES</t>
@@ -292,24 +373,48 @@
     <t>Fecha Inicio</t>
   </si>
   <si>
+    <t>01-05-2026 11:51:52</t>
+  </si>
+  <si>
+    <t>01-05-2026 12:28:55</t>
+  </si>
+  <si>
+    <t>01-05-2026 17:19:17</t>
+  </si>
+  <si>
+    <t>01-05-2026 18:12:55</t>
+  </si>
+  <si>
+    <t>14-04-2026 12:19:40</t>
+  </si>
+  <si>
+    <t>21-04-2026 13:16:43</t>
+  </si>
+  <si>
+    <t>24-04-2026 15:34:48</t>
+  </si>
+  <si>
+    <t>01-05-2026 10:34:42</t>
+  </si>
+  <si>
+    <t>01-05-2026 11:00:08</t>
+  </si>
+  <si>
+    <t>01-05-2026 11:42:18</t>
+  </si>
+  <si>
+    <t>01-05-2026 18:17:42</t>
+  </si>
+  <si>
+    <t>01-05-2026 18:32:13</t>
+  </si>
+  <si>
+    <t>02-05-2026 13:13:57</t>
+  </si>
+  <si>
     <t>31-03-2026 20:18:54</t>
   </si>
   <si>
-    <t>01-05-2026 10:34:42</t>
-  </si>
-  <si>
-    <t>01-05-2026 11:00:08</t>
-  </si>
-  <si>
-    <t>01-05-2026 11:42:18</t>
-  </si>
-  <si>
-    <t>01-05-2026 18:17:42</t>
-  </si>
-  <si>
-    <t>01-05-2026 18:32:13</t>
-  </si>
-  <si>
     <t>01-05-2026 9:28:55</t>
   </si>
   <si>
@@ -319,9 +424,42 @@
     <t>01-05-2026 17:35:18</t>
   </si>
   <si>
+    <t>02-05-2026 13:06:35</t>
+  </si>
+  <si>
     <t>10-04-2026 17:32:18</t>
   </si>
   <si>
+    <t>21-04-2026 13:14:32</t>
+  </si>
+  <si>
+    <t>02-04-2026 11:27:04</t>
+  </si>
+  <si>
+    <t>03-04-2026 10:04:26</t>
+  </si>
+  <si>
+    <t>06-04-2026 5:30:30</t>
+  </si>
+  <si>
+    <t>01-05-2026 10:38:33</t>
+  </si>
+  <si>
+    <t>01-05-2026 11:15:25</t>
+  </si>
+  <si>
+    <t>01-05-2026 19:13:51</t>
+  </si>
+  <si>
+    <t>02-05-2026 13:24:03</t>
+  </si>
+  <si>
+    <t>20-04-2026 20:14:31</t>
+  </si>
+  <si>
+    <t>04-03-2026 15:59:55</t>
+  </si>
+  <si>
     <t>27-04-2026 8:15:35</t>
   </si>
   <si>
@@ -334,19 +472,49 @@
     <t>01-05-2026 9:43:16</t>
   </si>
   <si>
+    <t>01-05-2026 20:01:10</t>
+  </si>
+  <si>
+    <t>01-05-2026 20:07:30</t>
+  </si>
+  <si>
     <t>11-04-2026 10:17:07</t>
   </si>
   <si>
-    <t>01-05-2026 11:51:52</t>
-  </si>
-  <si>
-    <t>01-05-2026 12:28:55</t>
-  </si>
-  <si>
-    <t>01-05-2026 17:19:17</t>
-  </si>
-  <si>
-    <t>01-05-2026 18:12:55</t>
+    <t>28-04-2026 13:00:52</t>
+  </si>
+  <si>
+    <t>24-03-2026 20:48:40</t>
+  </si>
+  <si>
+    <t>26-03-2026 13:42:06</t>
+  </si>
+  <si>
+    <t>01-05-2026 16:18:47</t>
+  </si>
+  <si>
+    <t>02-05-2026 7:36:52</t>
+  </si>
+  <si>
+    <t>03-04-2026 17:05:50</t>
+  </si>
+  <si>
+    <t>07-04-2026 17:54:05</t>
+  </si>
+  <si>
+    <t>20-04-2026 21:29:56</t>
+  </si>
+  <si>
+    <t>01-05-2026 10:01:13</t>
+  </si>
+  <si>
+    <t>01-05-2026 11:54:51</t>
+  </si>
+  <si>
+    <t>01-05-2026 16:31:24</t>
+  </si>
+  <si>
+    <t>01-05-2026 20:54:12</t>
   </si>
   <si>
     <t>02-04-2026 7:19:31</t>
@@ -355,40 +523,7 @@
     <t>02-04-2026 11:24:30</t>
   </si>
   <si>
-    <t>01-05-2026 10:01:13</t>
-  </si>
-  <si>
-    <t>01-05-2026 11:54:51</t>
-  </si>
-  <si>
-    <t>01-05-2026 16:31:24</t>
-  </si>
-  <si>
-    <t>28-04-2026 13:00:52</t>
-  </si>
-  <si>
-    <t>01-05-2026 16:18:47</t>
-  </si>
-  <si>
-    <t>26-03-2026 13:42:06</t>
-  </si>
-  <si>
-    <t>20-04-2026 21:29:56</t>
-  </si>
-  <si>
-    <t>02-04-2026 11:27:04</t>
-  </si>
-  <si>
-    <t>01-05-2026 10:38:33</t>
-  </si>
-  <si>
-    <t>01-05-2026 11:15:25</t>
-  </si>
-  <si>
-    <t>06-04-2026 5:30:30</t>
-  </si>
-  <si>
-    <t>20-04-2026 20:14:31</t>
+    <t>10-04-2026 15:14:18</t>
   </si>
   <si>
     <t>01-05-2026 7:38:40</t>
@@ -397,6 +532,9 @@
     <t>01-05-2026 8:37:34</t>
   </si>
   <si>
+    <t>02-05-2026 7:46:19</t>
+  </si>
+  <si>
     <t>08-04-2026 20:42:26</t>
   </si>
   <si>
@@ -412,9 +550,18 @@
     <t>30-05-2026 23:59:59</t>
   </si>
   <si>
+    <t>02-06-2026 23:59:59</t>
+  </si>
+  <si>
     <t>04-06-2026 23:59:59</t>
   </si>
   <si>
+    <t>03-05-2026 23:59:59</t>
+  </si>
+  <si>
+    <t>10-05-2026 23:59:59</t>
+  </si>
+  <si>
     <t>01-08-2026 23:59:59</t>
   </si>
   <si>
@@ -430,12 +577,12 @@
     <t>Estatus</t>
   </si>
   <si>
+    <t>NUEVO</t>
+  </si>
+  <si>
     <t>RENOVACIÓN</t>
   </si>
   <si>
-    <t>NUEVO</t>
-  </si>
-  <si>
     <t>Importe</t>
   </si>
   <si>
@@ -448,34 +595,97 @@
     <t>Fecha Fin Contrato</t>
   </si>
   <si>
+    <t>26-04-2027 12:28:55</t>
+  </si>
+  <si>
+    <t>28-10-2026 17:19:17</t>
+  </si>
+  <si>
+    <t>16-04-2027 13:16:43</t>
+  </si>
+  <si>
+    <t>21-10-2026 15:34:48</t>
+  </si>
+  <si>
+    <t>26-04-2027 10:34:42</t>
+  </si>
+  <si>
+    <t>26-04-2027 11:42:18</t>
+  </si>
+  <si>
+    <t>26-04-2027 18:17:42</t>
+  </si>
+  <si>
+    <t>26-04-2027 18:32:13</t>
+  </si>
+  <si>
     <t>26-03-2027 20:18:54</t>
   </si>
   <si>
-    <t>26-04-2027 10:34:42</t>
-  </si>
-  <si>
-    <t>26-04-2027 11:42:18</t>
-  </si>
-  <si>
-    <t>26-04-2027 18:17:42</t>
-  </si>
-  <si>
-    <t>26-04-2027 18:32:13</t>
-  </si>
-  <si>
     <t>26-04-2027 9:28:55</t>
   </si>
   <si>
     <t>26-04-2027 12:44:57</t>
   </si>
   <si>
+    <t>27-04-2027 13:06:35</t>
+  </si>
+  <si>
+    <t>16-04-2027 13:14:32</t>
+  </si>
+  <si>
+    <t>28-03-2027 11:27:04</t>
+  </si>
+  <si>
+    <t>30-09-2026 10:04:26</t>
+  </si>
+  <si>
+    <t>26-04-2027 11:15:25</t>
+  </si>
+  <si>
+    <t>27-04-2027 13:24:03</t>
+  </si>
+  <si>
+    <t>27-02-2027 15:59:55</t>
+  </si>
+  <si>
     <t>25-04-2027 8:06:02</t>
   </si>
   <si>
-    <t>26-04-2027 12:28:55</t>
-  </si>
-  <si>
-    <t>28-10-2026 17:19:17</t>
+    <t>26-04-2027 20:01:10</t>
+  </si>
+  <si>
+    <t>19-03-2027 20:48:40</t>
+  </si>
+  <si>
+    <t>21-03-2027 13:42:06</t>
+  </si>
+  <si>
+    <t>26-04-2027 16:18:47</t>
+  </si>
+  <si>
+    <t>27-04-2027 7:36:52</t>
+  </si>
+  <si>
+    <t>30-09-2026 17:05:50</t>
+  </si>
+  <si>
+    <t>02-04-2027 17:54:05</t>
+  </si>
+  <si>
+    <t>15-04-2027 21:29:56</t>
+  </si>
+  <si>
+    <t>26-04-2027 10:01:13</t>
+  </si>
+  <si>
+    <t>26-04-2027 11:54:51</t>
+  </si>
+  <si>
+    <t>26-04-2027 16:31:24</t>
+  </si>
+  <si>
+    <t>28-10-2026 20:54:12</t>
   </si>
   <si>
     <t>29-09-2026 7:19:31</t>
@@ -484,43 +694,22 @@
     <t>28-03-2027 11:24:30</t>
   </si>
   <si>
-    <t>26-04-2027 10:01:13</t>
-  </si>
-  <si>
-    <t>26-04-2027 11:54:51</t>
-  </si>
-  <si>
-    <t>26-04-2027 16:31:24</t>
-  </si>
-  <si>
-    <t>26-04-2027 16:18:47</t>
-  </si>
-  <si>
-    <t>21-03-2027 13:42:06</t>
-  </si>
-  <si>
-    <t>15-04-2027 21:29:56</t>
-  </si>
-  <si>
-    <t>28-03-2027 11:27:04</t>
-  </si>
-  <si>
-    <t>26-04-2027 11:15:25</t>
-  </si>
-  <si>
     <t>26-04-2027 8:37:34</t>
   </si>
   <si>
+    <t>27-04-2027 7:46:19</t>
+  </si>
+  <si>
     <t>26-04-2027 15:17:21</t>
   </si>
   <si>
     <t>Tipo Contrato</t>
   </si>
   <si>
+    <t>Recurrente</t>
+  </si>
+  <si>
     <t>Domiciliado</t>
-  </si>
-  <si>
-    <t>Recurrente</t>
   </si>
   <si>
     <t>Contrato Ajuste</t>
@@ -884,7 +1073,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:Q59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -951,43 +1140,43 @@
         <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="F2" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="G2" t="s">
-        <v>91</v>
+        <v>118</v>
       </c>
       <c r="H2" t="s">
-        <v>129</v>
+        <v>175</v>
       </c>
       <c r="I2" t="s">
-        <v>134</v>
+        <v>183</v>
       </c>
       <c r="J2" t="s">
-        <v>135</v>
+        <v>184</v>
       </c>
       <c r="K2" t="s">
-        <v>137</v>
+        <v>186</v>
       </c>
       <c r="L2" t="s">
-        <v>140</v>
+        <v>189</v>
       </c>
       <c r="M2" t="s">
-        <v>141</v>
+        <v>190</v>
       </c>
       <c r="N2" t="s">
-        <v>143</v>
+        <v>192</v>
       </c>
       <c r="O2" t="s">
-        <v>166</v>
+        <v>229</v>
       </c>
       <c r="P2" t="s">
-        <v>169</v>
+        <v>232</v>
       </c>
       <c r="Q2" t="s">
-        <v>170</v>
+        <v>233</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -995,49 +1184,43 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>98369</v>
+        <v>100493</v>
       </c>
       <c r="C3">
-        <v>56575</v>
-      </c>
-      <c r="D3">
-        <v>54426</v>
+        <v>360045</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F3" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="G3" t="s">
-        <v>92</v>
+        <v>119</v>
       </c>
       <c r="H3" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K3" t="s">
-        <v>138</v>
+        <v>187</v>
       </c>
       <c r="L3">
-        <v>499</v>
-      </c>
-      <c r="M3">
-        <v>11</v>
-      </c>
-      <c r="N3" t="s">
-        <v>144</v>
+        <v>799</v>
+      </c>
+      <c r="M3" t="s">
+        <v>191</v>
       </c>
       <c r="O3" t="s">
-        <v>167</v>
-      </c>
-      <c r="P3">
-        <v>91270</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -1045,46 +1228,46 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>100488</v>
+        <v>100495</v>
       </c>
       <c r="C4">
-        <v>360887</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
+        <v>349026</v>
+      </c>
+      <c r="D4">
+        <v>91191</v>
       </c>
       <c r="E4" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F4" t="s">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G4" t="s">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="H4" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I4">
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K4" t="s">
-        <v>139</v>
+        <v>187</v>
       </c>
       <c r="L4">
-        <v>549</v>
+        <v>649</v>
       </c>
       <c r="M4">
         <v>11</v>
       </c>
       <c r="N4" t="s">
-        <v>145</v>
+        <v>193</v>
       </c>
       <c r="O4" t="s">
-        <v>167</v>
+        <v>231</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -1092,43 +1275,49 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>100490</v>
+        <v>100502</v>
       </c>
       <c r="C5">
-        <v>360892</v>
+        <v>205459</v>
       </c>
       <c r="D5" t="s">
         <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="F5" t="s">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="G5" t="s">
-        <v>94</v>
+        <v>121</v>
       </c>
       <c r="H5" t="s">
-        <v>130</v>
+        <v>177</v>
       </c>
       <c r="I5">
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K5" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="L5">
-        <v>649</v>
-      </c>
-      <c r="M5" t="s">
-        <v>142</v>
+        <v>399</v>
+      </c>
+      <c r="M5">
+        <v>5</v>
+      </c>
+      <c r="N5" t="s">
+        <v>194</v>
       </c>
       <c r="O5" t="s">
-        <v>168</v>
+        <v>231</v>
+      </c>
+      <c r="P5">
+        <v>38806</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -1136,46 +1325,43 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>100492</v>
+        <v>100504</v>
       </c>
       <c r="C6">
-        <v>360904</v>
+        <v>361003</v>
       </c>
       <c r="D6" t="s">
         <v>23</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="F6" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="G6" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H6" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I6">
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K6" t="s">
-        <v>139</v>
+        <v>187</v>
       </c>
       <c r="L6">
-        <v>549</v>
-      </c>
-      <c r="M6">
-        <v>11</v>
-      </c>
-      <c r="N6" t="s">
-        <v>146</v>
+        <v>649</v>
+      </c>
+      <c r="M6" t="s">
+        <v>191</v>
       </c>
       <c r="O6" t="s">
-        <v>167</v>
+        <v>230</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -1183,46 +1369,46 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>100505</v>
+        <v>99332</v>
       </c>
       <c r="C7">
-        <v>360757</v>
-      </c>
-      <c r="D7" t="s">
-        <v>24</v>
+        <v>257916</v>
+      </c>
+      <c r="D7">
+        <v>55420</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="F7" t="s">
-        <v>77</v>
+        <v>103</v>
       </c>
       <c r="G7" t="s">
-        <v>96</v>
+        <v>123</v>
       </c>
       <c r="H7" t="s">
-        <v>130</v>
+        <v>178</v>
       </c>
       <c r="I7">
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K7" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="L7">
-        <v>549</v>
-      </c>
-      <c r="M7">
-        <v>11</v>
-      </c>
-      <c r="N7" t="s">
-        <v>147</v>
+        <v>399</v>
+      </c>
+      <c r="M7" t="s">
+        <v>191</v>
       </c>
       <c r="O7" t="s">
-        <v>167</v>
+        <v>230</v>
+      </c>
+      <c r="P7">
+        <v>73999</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -1230,46 +1416,49 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>100507</v>
+        <v>99890</v>
       </c>
       <c r="C8">
-        <v>353643</v>
+        <v>34927</v>
       </c>
       <c r="D8">
-        <v>95807</v>
+        <v>32841</v>
       </c>
       <c r="E8" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="F8" t="s">
-        <v>78</v>
+        <v>104</v>
       </c>
       <c r="G8" t="s">
-        <v>97</v>
+        <v>124</v>
       </c>
       <c r="H8" t="s">
-        <v>130</v>
+        <v>178</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K8" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="L8">
-        <v>649</v>
+        <v>499</v>
       </c>
       <c r="M8">
         <v>11</v>
       </c>
       <c r="N8" t="s">
-        <v>148</v>
+        <v>195</v>
       </c>
       <c r="O8" t="s">
-        <v>167</v>
+        <v>231</v>
+      </c>
+      <c r="P8">
+        <v>95584</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -1277,49 +1466,49 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>100485</v>
+        <v>100107</v>
       </c>
       <c r="C9">
-        <v>283428</v>
-      </c>
-      <c r="D9">
-        <v>80929</v>
+        <v>312465</v>
+      </c>
+      <c r="D9" t="s">
+        <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="F9" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
       <c r="G9" t="s">
-        <v>98</v>
+        <v>125</v>
       </c>
       <c r="H9" t="s">
-        <v>130</v>
+        <v>178</v>
       </c>
       <c r="I9">
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K9" t="s">
-        <v>138</v>
+        <v>188</v>
       </c>
       <c r="L9">
-        <v>699</v>
+        <v>549</v>
       </c>
       <c r="M9">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N9" t="s">
-        <v>149</v>
+        <v>196</v>
       </c>
       <c r="O9" t="s">
-        <v>167</v>
+        <v>231</v>
       </c>
       <c r="P9">
-        <v>60636</v>
+        <v>77036</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -1327,49 +1516,46 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>100496</v>
+        <v>100488</v>
       </c>
       <c r="C10">
-        <v>241908</v>
-      </c>
-      <c r="D10">
-        <v>39413</v>
+        <v>360887</v>
+      </c>
+      <c r="D10" t="s">
+        <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="F10" t="s">
-        <v>74</v>
+        <v>105</v>
       </c>
       <c r="G10" t="s">
-        <v>99</v>
+        <v>126</v>
       </c>
       <c r="H10" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I10">
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K10" t="s">
-        <v>138</v>
+        <v>187</v>
       </c>
       <c r="L10">
-        <v>699</v>
+        <v>549</v>
       </c>
       <c r="M10">
         <v>11</v>
       </c>
       <c r="N10" t="s">
-        <v>150</v>
+        <v>197</v>
       </c>
       <c r="O10" t="s">
-        <v>167</v>
-      </c>
-      <c r="P10">
-        <v>54257</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -1377,43 +1563,43 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>100503</v>
+        <v>100490</v>
       </c>
       <c r="C11">
-        <v>360991</v>
+        <v>360892</v>
       </c>
       <c r="D11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E11" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="F11" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="G11" t="s">
-        <v>100</v>
+        <v>127</v>
       </c>
       <c r="H11" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I11">
         <v>0</v>
       </c>
       <c r="J11" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K11" t="s">
-        <v>139</v>
+        <v>187</v>
       </c>
       <c r="L11">
         <v>649</v>
       </c>
       <c r="M11" t="s">
-        <v>142</v>
+        <v>191</v>
       </c>
       <c r="O11" t="s">
-        <v>168</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -1421,46 +1607,46 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>99056</v>
+        <v>100492</v>
       </c>
       <c r="C12">
-        <v>76774</v>
-      </c>
-      <c r="D12">
-        <v>74576</v>
+        <v>360904</v>
+      </c>
+      <c r="D12" t="s">
+        <v>27</v>
       </c>
       <c r="E12" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="F12" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="G12" t="s">
-        <v>101</v>
+        <v>128</v>
       </c>
       <c r="H12" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I12">
         <v>0</v>
       </c>
       <c r="J12" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K12" t="s">
-        <v>138</v>
+        <v>187</v>
       </c>
       <c r="L12">
-        <v>399</v>
-      </c>
-      <c r="M12" t="s">
-        <v>142</v>
+        <v>549</v>
+      </c>
+      <c r="M12">
+        <v>11</v>
+      </c>
+      <c r="N12" t="s">
+        <v>198</v>
       </c>
       <c r="O12" t="s">
-        <v>168</v>
-      </c>
-      <c r="P12">
-        <v>24188</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -1468,46 +1654,46 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>100177</v>
+        <v>100505</v>
       </c>
       <c r="C13">
-        <v>194060</v>
-      </c>
-      <c r="D13">
-        <v>91567</v>
+        <v>360757</v>
+      </c>
+      <c r="D13" t="s">
+        <v>28</v>
       </c>
       <c r="E13" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="F13" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="G13" t="s">
-        <v>102</v>
+        <v>129</v>
       </c>
       <c r="H13" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I13">
         <v>0</v>
       </c>
       <c r="J13" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K13" t="s">
-        <v>138</v>
+        <v>187</v>
       </c>
       <c r="L13">
-        <v>499</v>
-      </c>
-      <c r="M13" t="s">
-        <v>142</v>
+        <v>549</v>
+      </c>
+      <c r="M13">
+        <v>11</v>
+      </c>
+      <c r="N13" t="s">
+        <v>199</v>
       </c>
       <c r="O13" t="s">
-        <v>168</v>
-      </c>
-      <c r="P13">
-        <v>4813</v>
+        <v>231</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -1515,46 +1701,46 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>100443</v>
+        <v>100507</v>
       </c>
       <c r="C14">
-        <v>354766</v>
+        <v>353643</v>
       </c>
       <c r="D14">
-        <v>96930</v>
+        <v>95807</v>
       </c>
       <c r="E14" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="F14" t="s">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="G14" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="H14" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I14">
         <v>0</v>
       </c>
       <c r="J14" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K14" t="s">
-        <v>139</v>
+        <v>187</v>
       </c>
       <c r="L14">
-        <v>549</v>
+        <v>649</v>
       </c>
       <c r="M14">
         <v>11</v>
       </c>
       <c r="N14" t="s">
-        <v>151</v>
+        <v>200</v>
       </c>
       <c r="O14" t="s">
-        <v>167</v>
+        <v>231</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -1562,43 +1748,43 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>100484</v>
+        <v>100522</v>
       </c>
       <c r="C15">
-        <v>42885</v>
-      </c>
-      <c r="D15">
-        <v>40755</v>
+        <v>360630</v>
+      </c>
+      <c r="D15" t="s">
+        <v>29</v>
       </c>
       <c r="E15" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="F15" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="G15" t="s">
-        <v>104</v>
+        <v>131</v>
       </c>
       <c r="H15" t="s">
-        <v>130</v>
+        <v>178</v>
       </c>
       <c r="I15">
         <v>0</v>
       </c>
       <c r="J15" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K15" t="s">
-        <v>139</v>
+        <v>187</v>
       </c>
       <c r="L15">
-        <v>649</v>
+        <v>549</v>
       </c>
       <c r="M15" t="s">
-        <v>142</v>
+        <v>191</v>
       </c>
       <c r="O15" t="s">
-        <v>168</v>
+        <v>230</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -1606,43 +1792,49 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>100486</v>
+        <v>98369</v>
       </c>
       <c r="C16">
-        <v>360869</v>
-      </c>
-      <c r="D16" t="s">
-        <v>26</v>
+        <v>56575</v>
+      </c>
+      <c r="D16">
+        <v>54426</v>
       </c>
       <c r="E16" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="F16" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="G16" t="s">
-        <v>105</v>
+        <v>132</v>
       </c>
       <c r="H16" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I16">
         <v>0</v>
       </c>
       <c r="J16" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K16" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="L16">
-        <v>649</v>
-      </c>
-      <c r="M16" t="s">
-        <v>142</v>
+        <v>499</v>
+      </c>
+      <c r="M16">
+        <v>11</v>
+      </c>
+      <c r="N16" t="s">
+        <v>201</v>
       </c>
       <c r="O16" t="s">
-        <v>168</v>
+        <v>231</v>
+      </c>
+      <c r="P16">
+        <v>91270</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -1650,46 +1842,49 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>99080</v>
+        <v>100485</v>
       </c>
       <c r="C17">
-        <v>326105</v>
+        <v>283428</v>
       </c>
       <c r="D17">
-        <v>23044</v>
+        <v>80929</v>
       </c>
       <c r="E17" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="F17" t="s">
-        <v>82</v>
+        <v>107</v>
       </c>
       <c r="G17" t="s">
-        <v>106</v>
+        <v>133</v>
       </c>
       <c r="H17" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I17">
         <v>0</v>
       </c>
       <c r="J17" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K17" t="s">
-        <v>138</v>
+        <v>188</v>
       </c>
       <c r="L17">
-        <v>599</v>
-      </c>
-      <c r="M17" t="s">
-        <v>142</v>
+        <v>699</v>
+      </c>
+      <c r="M17">
+        <v>11</v>
+      </c>
+      <c r="N17" t="s">
+        <v>202</v>
       </c>
       <c r="O17" t="s">
-        <v>168</v>
+        <v>231</v>
       </c>
       <c r="P17">
-        <v>83122</v>
+        <v>60636</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -1697,43 +1892,49 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>100493</v>
+        <v>100496</v>
       </c>
       <c r="C18">
-        <v>360045</v>
-      </c>
-      <c r="D18" t="s">
-        <v>27</v>
+        <v>241908</v>
+      </c>
+      <c r="D18">
+        <v>39413</v>
       </c>
       <c r="E18" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F18" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="G18" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="H18" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I18">
         <v>0</v>
       </c>
       <c r="J18" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K18" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="L18">
-        <v>799</v>
-      </c>
-      <c r="M18" t="s">
-        <v>142</v>
+        <v>699</v>
+      </c>
+      <c r="M18">
+        <v>11</v>
+      </c>
+      <c r="N18" t="s">
+        <v>203</v>
       </c>
       <c r="O18" t="s">
-        <v>168</v>
+        <v>231</v>
+      </c>
+      <c r="P18">
+        <v>54257</v>
       </c>
     </row>
     <row r="19" spans="1:16">
@@ -1741,46 +1942,43 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>100495</v>
+        <v>100503</v>
       </c>
       <c r="C19">
-        <v>349026</v>
-      </c>
-      <c r="D19">
-        <v>91191</v>
+        <v>360991</v>
+      </c>
+      <c r="D19" t="s">
+        <v>30</v>
       </c>
       <c r="E19" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="F19" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
       <c r="G19" t="s">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="H19" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I19">
         <v>0</v>
       </c>
       <c r="J19" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K19" t="s">
-        <v>139</v>
+        <v>187</v>
       </c>
       <c r="L19">
         <v>649</v>
       </c>
-      <c r="M19">
-        <v>11</v>
-      </c>
-      <c r="N19" t="s">
-        <v>152</v>
+      <c r="M19" t="s">
+        <v>191</v>
       </c>
       <c r="O19" t="s">
-        <v>167</v>
+        <v>230</v>
       </c>
     </row>
     <row r="20" spans="1:16">
@@ -1788,49 +1986,46 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>100502</v>
+        <v>100521</v>
       </c>
       <c r="C20">
-        <v>205459</v>
-      </c>
-      <c r="D20" t="s">
-        <v>28</v>
+        <v>266562</v>
+      </c>
+      <c r="D20">
+        <v>64066</v>
       </c>
       <c r="E20" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="F20" t="s">
-        <v>77</v>
+        <v>109</v>
       </c>
       <c r="G20" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="H20" t="s">
-        <v>131</v>
+        <v>178</v>
       </c>
       <c r="I20">
         <v>0</v>
       </c>
       <c r="J20" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K20" t="s">
-        <v>138</v>
+        <v>187</v>
       </c>
       <c r="L20">
-        <v>399</v>
+        <v>499</v>
       </c>
       <c r="M20">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="N20" t="s">
-        <v>153</v>
+        <v>204</v>
       </c>
       <c r="O20" t="s">
-        <v>167</v>
-      </c>
-      <c r="P20">
-        <v>38806</v>
+        <v>231</v>
       </c>
     </row>
     <row r="21" spans="1:16">
@@ -1838,43 +2033,46 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>100504</v>
+        <v>99056</v>
       </c>
       <c r="C21">
-        <v>361003</v>
-      </c>
-      <c r="D21" t="s">
-        <v>29</v>
+        <v>76774</v>
+      </c>
+      <c r="D21">
+        <v>74576</v>
       </c>
       <c r="E21" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="F21" t="s">
-        <v>74</v>
+        <v>108</v>
       </c>
       <c r="G21" t="s">
-        <v>110</v>
+        <v>137</v>
       </c>
       <c r="H21" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I21">
         <v>0</v>
       </c>
       <c r="J21" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K21" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="L21">
-        <v>649</v>
+        <v>399</v>
       </c>
       <c r="M21" t="s">
-        <v>142</v>
+        <v>191</v>
       </c>
       <c r="O21" t="s">
-        <v>168</v>
+        <v>230</v>
+      </c>
+      <c r="P21">
+        <v>24188</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -1882,49 +2080,49 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>98454</v>
+        <v>99889</v>
       </c>
       <c r="C22">
-        <v>65078</v>
+        <v>17586</v>
       </c>
       <c r="D22">
-        <v>62916</v>
+        <v>16499</v>
       </c>
       <c r="E22" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="F22" t="s">
-        <v>82</v>
+        <v>104</v>
       </c>
       <c r="G22" t="s">
-        <v>111</v>
+        <v>138</v>
       </c>
       <c r="H22" t="s">
-        <v>130</v>
+        <v>178</v>
       </c>
       <c r="I22">
         <v>0</v>
       </c>
       <c r="J22" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K22" t="s">
-        <v>138</v>
+        <v>188</v>
       </c>
       <c r="L22">
-        <v>350</v>
+        <v>499</v>
       </c>
       <c r="M22">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="N22" t="s">
-        <v>154</v>
+        <v>205</v>
       </c>
       <c r="O22" t="s">
-        <v>167</v>
+        <v>231</v>
       </c>
       <c r="P22">
-        <v>76842</v>
+        <v>95586</v>
       </c>
     </row>
     <row r="23" spans="1:16">
@@ -1932,34 +2130,34 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>98465</v>
+        <v>98466</v>
       </c>
       <c r="C23">
-        <v>312044</v>
+        <v>205081</v>
       </c>
       <c r="D23" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E23" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F23" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="G23" t="s">
-        <v>112</v>
+        <v>139</v>
       </c>
       <c r="H23" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I23">
         <v>0</v>
       </c>
       <c r="J23" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K23" t="s">
-        <v>138</v>
+        <v>188</v>
       </c>
       <c r="L23">
         <v>499</v>
@@ -1968,13 +2166,13 @@
         <v>11</v>
       </c>
       <c r="N23" t="s">
-        <v>155</v>
+        <v>206</v>
       </c>
       <c r="O23" t="s">
-        <v>167</v>
+        <v>231</v>
       </c>
       <c r="P23">
-        <v>76811</v>
+        <v>76809</v>
       </c>
     </row>
     <row r="24" spans="1:16">
@@ -1982,46 +2180,49 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>100487</v>
+        <v>98517</v>
       </c>
       <c r="C24">
-        <v>48666</v>
+        <v>232630</v>
       </c>
       <c r="D24">
-        <v>46524</v>
+        <v>30135</v>
       </c>
       <c r="E24" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="F24" t="s">
-        <v>84</v>
+        <v>109</v>
       </c>
       <c r="G24" t="s">
-        <v>113</v>
+        <v>140</v>
       </c>
       <c r="H24" t="s">
-        <v>130</v>
+        <v>178</v>
       </c>
       <c r="I24">
         <v>0</v>
       </c>
       <c r="J24" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K24" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="L24">
-        <v>549</v>
+        <v>449</v>
       </c>
       <c r="M24">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N24" t="s">
-        <v>156</v>
+        <v>207</v>
       </c>
       <c r="O24" t="s">
-        <v>167</v>
+        <v>231</v>
+      </c>
+      <c r="P24">
+        <v>49260</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -2029,46 +2230,46 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>100494</v>
+        <v>98583</v>
       </c>
       <c r="C25">
-        <v>346010</v>
+        <v>114721</v>
       </c>
       <c r="D25">
-        <v>88175</v>
+        <v>12446</v>
       </c>
       <c r="E25" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F25" t="s">
-        <v>79</v>
+        <v>110</v>
       </c>
       <c r="G25" t="s">
-        <v>114</v>
+        <v>141</v>
       </c>
       <c r="H25" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I25">
         <v>0</v>
       </c>
       <c r="J25" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K25" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="L25">
-        <v>999</v>
-      </c>
-      <c r="M25">
-        <v>11</v>
-      </c>
-      <c r="N25" t="s">
-        <v>157</v>
+        <v>399</v>
+      </c>
+      <c r="M25" t="s">
+        <v>191</v>
       </c>
       <c r="O25" t="s">
-        <v>167</v>
+        <v>230</v>
+      </c>
+      <c r="P25">
+        <v>11835</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -2076,46 +2277,43 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>100501</v>
+        <v>100489</v>
       </c>
       <c r="C26">
-        <v>347090</v>
-      </c>
-      <c r="D26">
-        <v>89255</v>
+        <v>360888</v>
+      </c>
+      <c r="D26" t="s">
+        <v>32</v>
       </c>
       <c r="E26" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F26" t="s">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="G26" t="s">
-        <v>115</v>
+        <v>142</v>
       </c>
       <c r="H26" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I26">
         <v>0</v>
       </c>
       <c r="J26" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K26" t="s">
-        <v>139</v>
+        <v>187</v>
       </c>
       <c r="L26">
-        <v>549</v>
-      </c>
-      <c r="M26">
-        <v>11</v>
-      </c>
-      <c r="N26" t="s">
-        <v>158</v>
+        <v>649</v>
+      </c>
+      <c r="M26" t="s">
+        <v>191</v>
       </c>
       <c r="O26" t="s">
-        <v>167</v>
+        <v>230</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -2123,46 +2321,49 @@
         <v>25</v>
       </c>
       <c r="B27">
-        <v>100331</v>
+        <v>100491</v>
       </c>
       <c r="C27">
-        <v>22791</v>
+        <v>56971</v>
       </c>
       <c r="D27">
-        <v>21685</v>
+        <v>54822</v>
       </c>
       <c r="E27" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="F27" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="G27" t="s">
-        <v>116</v>
+        <v>143</v>
       </c>
       <c r="H27" t="s">
-        <v>130</v>
+        <v>179</v>
       </c>
       <c r="I27">
         <v>0</v>
       </c>
       <c r="J27" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K27" t="s">
-        <v>138</v>
+        <v>188</v>
       </c>
       <c r="L27">
-        <v>399</v>
-      </c>
-      <c r="M27" t="s">
-        <v>142</v>
+        <v>449</v>
+      </c>
+      <c r="M27">
+        <v>11</v>
+      </c>
+      <c r="N27" t="s">
+        <v>208</v>
       </c>
       <c r="O27" t="s">
-        <v>168</v>
+        <v>231</v>
       </c>
       <c r="P27">
-        <v>79141</v>
+        <v>68495</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -2170,46 +2371,43 @@
         <v>26</v>
       </c>
       <c r="B28">
-        <v>100499</v>
+        <v>100508</v>
       </c>
       <c r="C28">
-        <v>79792</v>
-      </c>
-      <c r="D28">
-        <v>77591</v>
+        <v>361018</v>
+      </c>
+      <c r="D28" t="s">
+        <v>33</v>
       </c>
       <c r="E28" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F28" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="G28" t="s">
-        <v>117</v>
+        <v>144</v>
       </c>
       <c r="H28" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I28">
         <v>0</v>
       </c>
       <c r="J28" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K28" t="s">
-        <v>139</v>
+        <v>187</v>
       </c>
       <c r="L28">
-        <v>549</v>
-      </c>
-      <c r="M28">
-        <v>11</v>
-      </c>
-      <c r="N28" t="s">
-        <v>159</v>
+        <v>649</v>
+      </c>
+      <c r="M28" t="s">
+        <v>191</v>
       </c>
       <c r="O28" t="s">
-        <v>167</v>
+        <v>230</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -2217,49 +2415,49 @@
         <v>27</v>
       </c>
       <c r="B29">
-        <v>97892</v>
+        <v>100523</v>
       </c>
       <c r="C29">
-        <v>151685</v>
+        <v>177956</v>
       </c>
       <c r="D29">
-        <v>49250</v>
+        <v>75463</v>
       </c>
       <c r="E29" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="F29" t="s">
-        <v>82</v>
+        <v>107</v>
       </c>
       <c r="G29" t="s">
-        <v>118</v>
+        <v>145</v>
       </c>
       <c r="H29" t="s">
-        <v>130</v>
+        <v>178</v>
       </c>
       <c r="I29">
         <v>0</v>
       </c>
       <c r="J29" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K29" t="s">
-        <v>138</v>
+        <v>188</v>
       </c>
       <c r="L29">
-        <v>399</v>
+        <v>499</v>
       </c>
       <c r="M29">
         <v>11</v>
       </c>
       <c r="N29" t="s">
-        <v>160</v>
+        <v>209</v>
       </c>
       <c r="O29" t="s">
-        <v>167</v>
+        <v>231</v>
       </c>
       <c r="P29">
-        <v>2308</v>
+        <v>4701</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -2267,49 +2465,46 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>99846</v>
+        <v>99840</v>
       </c>
       <c r="C30">
-        <v>253406</v>
+        <v>178067</v>
       </c>
       <c r="D30">
-        <v>50910</v>
+        <v>75574</v>
       </c>
       <c r="E30" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F30" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="G30" t="s">
-        <v>119</v>
+        <v>146</v>
       </c>
       <c r="H30" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I30">
         <v>0</v>
       </c>
       <c r="J30" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K30" t="s">
-        <v>138</v>
+        <v>188</v>
       </c>
       <c r="L30">
-        <v>499</v>
-      </c>
-      <c r="M30">
-        <v>11</v>
-      </c>
-      <c r="N30" t="s">
-        <v>161</v>
+        <v>449</v>
+      </c>
+      <c r="M30" t="s">
+        <v>191</v>
       </c>
       <c r="O30" t="s">
-        <v>167</v>
+        <v>230</v>
       </c>
       <c r="P30">
-        <v>79273</v>
+        <v>74406</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -2317,34 +2512,34 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>98466</v>
+        <v>95940</v>
       </c>
       <c r="C31">
-        <v>205081</v>
-      </c>
-      <c r="D31" t="s">
-        <v>31</v>
+        <v>95151</v>
+      </c>
+      <c r="D31">
+        <v>92910</v>
       </c>
       <c r="E31" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F31" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="G31" t="s">
-        <v>120</v>
+        <v>147</v>
       </c>
       <c r="H31" t="s">
-        <v>130</v>
+        <v>180</v>
       </c>
       <c r="I31">
         <v>0</v>
       </c>
       <c r="J31" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K31" t="s">
-        <v>138</v>
+        <v>188</v>
       </c>
       <c r="L31">
         <v>499</v>
@@ -2353,13 +2548,13 @@
         <v>11</v>
       </c>
       <c r="N31" t="s">
-        <v>162</v>
+        <v>210</v>
       </c>
       <c r="O31" t="s">
-        <v>167</v>
+        <v>231</v>
       </c>
       <c r="P31">
-        <v>76809</v>
+        <v>52003</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -2367,43 +2562,46 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>100489</v>
+        <v>100177</v>
       </c>
       <c r="C32">
-        <v>360888</v>
-      </c>
-      <c r="D32" t="s">
-        <v>32</v>
+        <v>194060</v>
+      </c>
+      <c r="D32">
+        <v>91567</v>
       </c>
       <c r="E32" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="F32" t="s">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="G32" t="s">
-        <v>121</v>
+        <v>148</v>
       </c>
       <c r="H32" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I32">
         <v>0</v>
       </c>
       <c r="J32" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K32" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="L32">
-        <v>649</v>
+        <v>499</v>
       </c>
       <c r="M32" t="s">
-        <v>142</v>
+        <v>191</v>
       </c>
       <c r="O32" t="s">
-        <v>168</v>
+        <v>230</v>
+      </c>
+      <c r="P32">
+        <v>4813</v>
       </c>
     </row>
     <row r="33" spans="1:16">
@@ -2411,49 +2609,46 @@
         <v>31</v>
       </c>
       <c r="B33">
-        <v>100491</v>
+        <v>100443</v>
       </c>
       <c r="C33">
-        <v>56971</v>
+        <v>354766</v>
       </c>
       <c r="D33">
-        <v>54822</v>
+        <v>96930</v>
       </c>
       <c r="E33" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F33" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="G33" t="s">
-        <v>122</v>
+        <v>149</v>
       </c>
       <c r="H33" t="s">
-        <v>132</v>
+        <v>176</v>
       </c>
       <c r="I33">
         <v>0</v>
       </c>
       <c r="J33" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K33" t="s">
-        <v>138</v>
+        <v>187</v>
       </c>
       <c r="L33">
-        <v>449</v>
+        <v>549</v>
       </c>
       <c r="M33">
         <v>11</v>
       </c>
       <c r="N33" t="s">
-        <v>163</v>
+        <v>211</v>
       </c>
       <c r="O33" t="s">
-        <v>167</v>
-      </c>
-      <c r="P33">
-        <v>68495</v>
+        <v>231</v>
       </c>
     </row>
     <row r="34" spans="1:16">
@@ -2461,46 +2656,43 @@
         <v>32</v>
       </c>
       <c r="B34">
-        <v>98583</v>
+        <v>100484</v>
       </c>
       <c r="C34">
-        <v>114721</v>
+        <v>42885</v>
       </c>
       <c r="D34">
-        <v>12446</v>
+        <v>40755</v>
       </c>
       <c r="E34" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="F34" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="G34" t="s">
-        <v>123</v>
+        <v>150</v>
       </c>
       <c r="H34" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I34">
         <v>0</v>
       </c>
       <c r="J34" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K34" t="s">
-        <v>138</v>
+        <v>187</v>
       </c>
       <c r="L34">
-        <v>399</v>
+        <v>649</v>
       </c>
       <c r="M34" t="s">
-        <v>142</v>
+        <v>191</v>
       </c>
       <c r="O34" t="s">
-        <v>168</v>
-      </c>
-      <c r="P34">
-        <v>11835</v>
+        <v>230</v>
       </c>
     </row>
     <row r="35" spans="1:16">
@@ -2508,46 +2700,43 @@
         <v>33</v>
       </c>
       <c r="B35">
-        <v>99840</v>
+        <v>100486</v>
       </c>
       <c r="C35">
-        <v>178067</v>
-      </c>
-      <c r="D35">
-        <v>75574</v>
+        <v>360869</v>
+      </c>
+      <c r="D35" t="s">
+        <v>34</v>
       </c>
       <c r="E35" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F35" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="G35" t="s">
-        <v>124</v>
+        <v>151</v>
       </c>
       <c r="H35" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I35">
         <v>0</v>
       </c>
       <c r="J35" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K35" t="s">
-        <v>138</v>
+        <v>187</v>
       </c>
       <c r="L35">
-        <v>449</v>
+        <v>649</v>
       </c>
       <c r="M35" t="s">
-        <v>142</v>
+        <v>191</v>
       </c>
       <c r="O35" t="s">
-        <v>168</v>
-      </c>
-      <c r="P35">
-        <v>74406</v>
+        <v>230</v>
       </c>
     </row>
     <row r="36" spans="1:16">
@@ -2555,43 +2744,49 @@
         <v>34</v>
       </c>
       <c r="B36">
-        <v>100480</v>
+        <v>100509</v>
       </c>
       <c r="C36">
-        <v>360840</v>
-      </c>
-      <c r="D36" t="s">
-        <v>33</v>
+        <v>141351</v>
+      </c>
+      <c r="D36">
+        <v>38969</v>
       </c>
       <c r="E36" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="F36" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="G36" t="s">
-        <v>125</v>
+        <v>152</v>
       </c>
       <c r="H36" t="s">
-        <v>133</v>
+        <v>176</v>
       </c>
       <c r="I36">
         <v>0</v>
       </c>
       <c r="J36" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K36" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="L36">
-        <v>1549</v>
-      </c>
-      <c r="M36" t="s">
-        <v>142</v>
+        <v>699</v>
+      </c>
+      <c r="M36">
+        <v>11</v>
+      </c>
+      <c r="N36" t="s">
+        <v>212</v>
       </c>
       <c r="O36" t="s">
-        <v>168</v>
+        <v>231</v>
+      </c>
+      <c r="P36">
+        <v>76258</v>
       </c>
     </row>
     <row r="37" spans="1:16">
@@ -2599,46 +2794,43 @@
         <v>35</v>
       </c>
       <c r="B37">
-        <v>100483</v>
+        <v>100511</v>
       </c>
       <c r="C37">
-        <v>360852</v>
+        <v>361026</v>
       </c>
       <c r="D37" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E37" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="F37" t="s">
-        <v>83</v>
+        <v>109</v>
       </c>
       <c r="G37" t="s">
-        <v>126</v>
+        <v>153</v>
       </c>
       <c r="H37" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I37">
         <v>0</v>
       </c>
       <c r="J37" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K37" t="s">
-        <v>139</v>
+        <v>187</v>
       </c>
       <c r="L37">
         <v>649</v>
       </c>
-      <c r="M37">
-        <v>11</v>
-      </c>
-      <c r="N37" t="s">
-        <v>164</v>
+      <c r="M37" t="s">
+        <v>191</v>
       </c>
       <c r="O37" t="s">
-        <v>167</v>
+        <v>230</v>
       </c>
     </row>
     <row r="38" spans="1:16">
@@ -2646,46 +2838,46 @@
         <v>36</v>
       </c>
       <c r="B38">
-        <v>98943</v>
+        <v>99080</v>
       </c>
       <c r="C38">
-        <v>37106</v>
+        <v>326105</v>
       </c>
       <c r="D38">
-        <v>34985</v>
+        <v>23044</v>
       </c>
       <c r="E38" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F38" t="s">
-        <v>77</v>
+        <v>103</v>
       </c>
       <c r="G38" t="s">
-        <v>127</v>
+        <v>154</v>
       </c>
       <c r="H38" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="I38">
         <v>0</v>
       </c>
       <c r="J38" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="K38" t="s">
-        <v>138</v>
+        <v>188</v>
       </c>
       <c r="L38">
-        <v>399</v>
+        <v>599</v>
       </c>
       <c r="M38" t="s">
-        <v>142</v>
+        <v>191</v>
       </c>
       <c r="O38" t="s">
-        <v>168</v>
+        <v>230</v>
       </c>
       <c r="P38">
-        <v>96274</v>
+        <v>83122</v>
       </c>
     </row>
     <row r="39" spans="1:16">
@@ -2693,53 +2885,967 @@
         <v>37</v>
       </c>
       <c r="B39">
+        <v>100331</v>
+      </c>
+      <c r="C39">
+        <v>22791</v>
+      </c>
+      <c r="D39">
+        <v>21685</v>
+      </c>
+      <c r="E39" t="s">
+        <v>78</v>
+      </c>
+      <c r="F39" t="s">
+        <v>109</v>
+      </c>
+      <c r="G39" t="s">
+        <v>155</v>
+      </c>
+      <c r="H39" t="s">
+        <v>176</v>
+      </c>
+      <c r="I39">
+        <v>0</v>
+      </c>
+      <c r="J39" t="s">
+        <v>185</v>
+      </c>
+      <c r="K39" t="s">
+        <v>188</v>
+      </c>
+      <c r="L39">
+        <v>399</v>
+      </c>
+      <c r="M39" t="s">
+        <v>191</v>
+      </c>
+      <c r="O39" t="s">
+        <v>230</v>
+      </c>
+      <c r="P39">
+        <v>79141</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16">
+      <c r="A40">
+        <v>38</v>
+      </c>
+      <c r="B40">
+        <v>97773</v>
+      </c>
+      <c r="C40">
+        <v>348244</v>
+      </c>
+      <c r="D40">
+        <v>90409</v>
+      </c>
+      <c r="E40" t="s">
+        <v>79</v>
+      </c>
+      <c r="F40" t="s">
+        <v>102</v>
+      </c>
+      <c r="G40" t="s">
+        <v>156</v>
+      </c>
+      <c r="H40" t="s">
+        <v>181</v>
+      </c>
+      <c r="I40">
+        <v>0</v>
+      </c>
+      <c r="J40" t="s">
+        <v>185</v>
+      </c>
+      <c r="K40" t="s">
+        <v>188</v>
+      </c>
+      <c r="L40">
+        <v>549</v>
+      </c>
+      <c r="M40">
+        <v>11</v>
+      </c>
+      <c r="N40" t="s">
+        <v>213</v>
+      </c>
+      <c r="O40" t="s">
+        <v>231</v>
+      </c>
+      <c r="P40">
+        <v>97756</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16">
+      <c r="A41">
+        <v>39</v>
+      </c>
+      <c r="B41">
+        <v>97892</v>
+      </c>
+      <c r="C41">
+        <v>151685</v>
+      </c>
+      <c r="D41">
+        <v>49250</v>
+      </c>
+      <c r="E41" t="s">
+        <v>80</v>
+      </c>
+      <c r="F41" t="s">
+        <v>103</v>
+      </c>
+      <c r="G41" t="s">
+        <v>157</v>
+      </c>
+      <c r="H41" t="s">
+        <v>176</v>
+      </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
+      <c r="J41" t="s">
+        <v>185</v>
+      </c>
+      <c r="K41" t="s">
+        <v>188</v>
+      </c>
+      <c r="L41">
+        <v>399</v>
+      </c>
+      <c r="M41">
+        <v>11</v>
+      </c>
+      <c r="N41" t="s">
+        <v>214</v>
+      </c>
+      <c r="O41" t="s">
+        <v>231</v>
+      </c>
+      <c r="P41">
+        <v>2308</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16">
+      <c r="A42">
+        <v>40</v>
+      </c>
+      <c r="B42">
+        <v>100499</v>
+      </c>
+      <c r="C42">
+        <v>79792</v>
+      </c>
+      <c r="D42">
+        <v>77591</v>
+      </c>
+      <c r="E42" t="s">
+        <v>81</v>
+      </c>
+      <c r="F42" t="s">
+        <v>112</v>
+      </c>
+      <c r="G42" t="s">
+        <v>158</v>
+      </c>
+      <c r="H42" t="s">
+        <v>176</v>
+      </c>
+      <c r="I42">
+        <v>0</v>
+      </c>
+      <c r="J42" t="s">
+        <v>185</v>
+      </c>
+      <c r="K42" t="s">
+        <v>187</v>
+      </c>
+      <c r="L42">
+        <v>549</v>
+      </c>
+      <c r="M42">
+        <v>11</v>
+      </c>
+      <c r="N42" t="s">
+        <v>215</v>
+      </c>
+      <c r="O42" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16">
+      <c r="A43">
+        <v>41</v>
+      </c>
+      <c r="B43">
+        <v>100514</v>
+      </c>
+      <c r="C43">
+        <v>361054</v>
+      </c>
+      <c r="D43" t="s">
+        <v>36</v>
+      </c>
+      <c r="E43" t="s">
+        <v>82</v>
+      </c>
+      <c r="F43" t="s">
+        <v>100</v>
+      </c>
+      <c r="G43" t="s">
+        <v>159</v>
+      </c>
+      <c r="H43" t="s">
+        <v>178</v>
+      </c>
+      <c r="I43">
+        <v>0</v>
+      </c>
+      <c r="J43" t="s">
+        <v>185</v>
+      </c>
+      <c r="K43" t="s">
+        <v>187</v>
+      </c>
+      <c r="L43">
+        <v>649</v>
+      </c>
+      <c r="M43">
+        <v>11</v>
+      </c>
+      <c r="N43" t="s">
+        <v>216</v>
+      </c>
+      <c r="O43" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16">
+      <c r="A44">
+        <v>42</v>
+      </c>
+      <c r="B44">
+        <v>98541</v>
+      </c>
+      <c r="C44">
+        <v>25207</v>
+      </c>
+      <c r="D44">
+        <v>23149</v>
+      </c>
+      <c r="E44" t="s">
+        <v>83</v>
+      </c>
+      <c r="F44" t="s">
+        <v>109</v>
+      </c>
+      <c r="G44" t="s">
+        <v>160</v>
+      </c>
+      <c r="H44" t="s">
+        <v>178</v>
+      </c>
+      <c r="I44">
+        <v>0</v>
+      </c>
+      <c r="J44" t="s">
+        <v>185</v>
+      </c>
+      <c r="K44" t="s">
+        <v>188</v>
+      </c>
+      <c r="L44">
+        <v>449</v>
+      </c>
+      <c r="M44">
+        <v>5</v>
+      </c>
+      <c r="N44" t="s">
+        <v>217</v>
+      </c>
+      <c r="O44" t="s">
+        <v>231</v>
+      </c>
+      <c r="P44">
+        <v>49403</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16">
+      <c r="A45">
+        <v>43</v>
+      </c>
+      <c r="B45">
+        <v>98810</v>
+      </c>
+      <c r="C45">
+        <v>59822</v>
+      </c>
+      <c r="D45">
+        <v>57663</v>
+      </c>
+      <c r="E45" t="s">
+        <v>84</v>
+      </c>
+      <c r="F45" t="s">
+        <v>113</v>
+      </c>
+      <c r="G45" t="s">
+        <v>161</v>
+      </c>
+      <c r="H45" t="s">
+        <v>178</v>
+      </c>
+      <c r="I45">
+        <v>0</v>
+      </c>
+      <c r="J45" t="s">
+        <v>185</v>
+      </c>
+      <c r="K45" t="s">
+        <v>188</v>
+      </c>
+      <c r="L45">
+        <v>399</v>
+      </c>
+      <c r="M45">
+        <v>11</v>
+      </c>
+      <c r="N45" t="s">
+        <v>218</v>
+      </c>
+      <c r="O45" t="s">
+        <v>231</v>
+      </c>
+      <c r="P45">
+        <v>8024</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16">
+      <c r="A46">
+        <v>44</v>
+      </c>
+      <c r="B46">
+        <v>99846</v>
+      </c>
+      <c r="C46">
+        <v>253406</v>
+      </c>
+      <c r="D46">
+        <v>50910</v>
+      </c>
+      <c r="E46" t="s">
+        <v>85</v>
+      </c>
+      <c r="F46" t="s">
+        <v>114</v>
+      </c>
+      <c r="G46" t="s">
+        <v>162</v>
+      </c>
+      <c r="H46" t="s">
+        <v>176</v>
+      </c>
+      <c r="I46">
+        <v>0</v>
+      </c>
+      <c r="J46" t="s">
+        <v>185</v>
+      </c>
+      <c r="K46" t="s">
+        <v>188</v>
+      </c>
+      <c r="L46">
+        <v>499</v>
+      </c>
+      <c r="M46">
+        <v>11</v>
+      </c>
+      <c r="N46" t="s">
+        <v>219</v>
+      </c>
+      <c r="O46" t="s">
+        <v>231</v>
+      </c>
+      <c r="P46">
+        <v>79273</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16">
+      <c r="A47">
+        <v>45</v>
+      </c>
+      <c r="B47">
+        <v>100487</v>
+      </c>
+      <c r="C47">
+        <v>48666</v>
+      </c>
+      <c r="D47">
+        <v>46524</v>
+      </c>
+      <c r="E47" t="s">
+        <v>86</v>
+      </c>
+      <c r="F47" t="s">
+        <v>115</v>
+      </c>
+      <c r="G47" t="s">
+        <v>163</v>
+      </c>
+      <c r="H47" t="s">
+        <v>176</v>
+      </c>
+      <c r="I47">
+        <v>0</v>
+      </c>
+      <c r="J47" t="s">
+        <v>185</v>
+      </c>
+      <c r="K47" t="s">
+        <v>187</v>
+      </c>
+      <c r="L47">
+        <v>549</v>
+      </c>
+      <c r="M47">
+        <v>11</v>
+      </c>
+      <c r="N47" t="s">
+        <v>220</v>
+      </c>
+      <c r="O47" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16">
+      <c r="A48">
+        <v>46</v>
+      </c>
+      <c r="B48">
+        <v>100494</v>
+      </c>
+      <c r="C48">
+        <v>346010</v>
+      </c>
+      <c r="D48">
+        <v>88175</v>
+      </c>
+      <c r="E48" t="s">
+        <v>87</v>
+      </c>
+      <c r="F48" t="s">
+        <v>107</v>
+      </c>
+      <c r="G48" t="s">
+        <v>164</v>
+      </c>
+      <c r="H48" t="s">
+        <v>176</v>
+      </c>
+      <c r="I48">
+        <v>0</v>
+      </c>
+      <c r="J48" t="s">
+        <v>185</v>
+      </c>
+      <c r="K48" t="s">
+        <v>187</v>
+      </c>
+      <c r="L48">
+        <v>999</v>
+      </c>
+      <c r="M48">
+        <v>11</v>
+      </c>
+      <c r="N48" t="s">
+        <v>221</v>
+      </c>
+      <c r="O48" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16">
+      <c r="A49">
+        <v>47</v>
+      </c>
+      <c r="B49">
+        <v>100501</v>
+      </c>
+      <c r="C49">
+        <v>347090</v>
+      </c>
+      <c r="D49">
+        <v>89255</v>
+      </c>
+      <c r="E49" t="s">
+        <v>88</v>
+      </c>
+      <c r="F49" t="s">
+        <v>101</v>
+      </c>
+      <c r="G49" t="s">
+        <v>165</v>
+      </c>
+      <c r="H49" t="s">
+        <v>176</v>
+      </c>
+      <c r="I49">
+        <v>0</v>
+      </c>
+      <c r="J49" t="s">
+        <v>185</v>
+      </c>
+      <c r="K49" t="s">
+        <v>187</v>
+      </c>
+      <c r="L49">
+        <v>549</v>
+      </c>
+      <c r="M49">
+        <v>11</v>
+      </c>
+      <c r="N49" t="s">
+        <v>222</v>
+      </c>
+      <c r="O49" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16">
+      <c r="A50">
+        <v>48</v>
+      </c>
+      <c r="B50">
+        <v>100512</v>
+      </c>
+      <c r="C50">
+        <v>140437</v>
+      </c>
+      <c r="D50">
+        <v>38064</v>
+      </c>
+      <c r="E50" t="s">
+        <v>89</v>
+      </c>
+      <c r="F50" t="s">
+        <v>115</v>
+      </c>
+      <c r="G50" t="s">
+        <v>166</v>
+      </c>
+      <c r="H50" t="s">
+        <v>179</v>
+      </c>
+      <c r="I50">
+        <v>0</v>
+      </c>
+      <c r="J50" t="s">
+        <v>185</v>
+      </c>
+      <c r="K50" t="s">
+        <v>188</v>
+      </c>
+      <c r="L50">
+        <v>449</v>
+      </c>
+      <c r="M50">
+        <v>5</v>
+      </c>
+      <c r="N50" t="s">
+        <v>223</v>
+      </c>
+      <c r="O50" t="s">
+        <v>231</v>
+      </c>
+      <c r="P50">
+        <v>55808</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16">
+      <c r="A51">
+        <v>49</v>
+      </c>
+      <c r="B51">
+        <v>98454</v>
+      </c>
+      <c r="C51">
+        <v>65078</v>
+      </c>
+      <c r="D51">
+        <v>62916</v>
+      </c>
+      <c r="E51" t="s">
+        <v>90</v>
+      </c>
+      <c r="F51" t="s">
+        <v>103</v>
+      </c>
+      <c r="G51" t="s">
+        <v>167</v>
+      </c>
+      <c r="H51" t="s">
+        <v>176</v>
+      </c>
+      <c r="I51">
+        <v>0</v>
+      </c>
+      <c r="J51" t="s">
+        <v>185</v>
+      </c>
+      <c r="K51" t="s">
+        <v>188</v>
+      </c>
+      <c r="L51">
+        <v>350</v>
+      </c>
+      <c r="M51">
+        <v>5</v>
+      </c>
+      <c r="N51" t="s">
+        <v>224</v>
+      </c>
+      <c r="O51" t="s">
+        <v>231</v>
+      </c>
+      <c r="P51">
+        <v>76842</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16">
+      <c r="A52">
+        <v>50</v>
+      </c>
+      <c r="B52">
+        <v>98465</v>
+      </c>
+      <c r="C52">
+        <v>312044</v>
+      </c>
+      <c r="D52" t="s">
+        <v>37</v>
+      </c>
+      <c r="E52" t="s">
+        <v>91</v>
+      </c>
+      <c r="F52" t="s">
+        <v>104</v>
+      </c>
+      <c r="G52" t="s">
+        <v>168</v>
+      </c>
+      <c r="H52" t="s">
+        <v>176</v>
+      </c>
+      <c r="I52">
+        <v>0</v>
+      </c>
+      <c r="J52" t="s">
+        <v>185</v>
+      </c>
+      <c r="K52" t="s">
+        <v>188</v>
+      </c>
+      <c r="L52">
+        <v>499</v>
+      </c>
+      <c r="M52">
+        <v>11</v>
+      </c>
+      <c r="N52" t="s">
+        <v>225</v>
+      </c>
+      <c r="O52" t="s">
+        <v>231</v>
+      </c>
+      <c r="P52">
+        <v>76811</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16">
+      <c r="A53">
+        <v>51</v>
+      </c>
+      <c r="B53">
+        <v>99047</v>
+      </c>
+      <c r="C53">
+        <v>38715</v>
+      </c>
+      <c r="D53">
+        <v>36587</v>
+      </c>
+      <c r="E53" t="s">
+        <v>92</v>
+      </c>
+      <c r="F53" t="s">
+        <v>116</v>
+      </c>
+      <c r="G53" t="s">
+        <v>169</v>
+      </c>
+      <c r="H53" t="s">
+        <v>178</v>
+      </c>
+      <c r="I53">
+        <v>0</v>
+      </c>
+      <c r="J53" t="s">
+        <v>185</v>
+      </c>
+      <c r="K53" t="s">
+        <v>188</v>
+      </c>
+      <c r="L53">
+        <v>399</v>
+      </c>
+      <c r="M53" t="s">
+        <v>191</v>
+      </c>
+      <c r="O53" t="s">
+        <v>230</v>
+      </c>
+      <c r="P53">
+        <v>57290</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16">
+      <c r="A54">
+        <v>52</v>
+      </c>
+      <c r="B54">
+        <v>100480</v>
+      </c>
+      <c r="C54">
+        <v>360840</v>
+      </c>
+      <c r="D54" t="s">
+        <v>38</v>
+      </c>
+      <c r="E54" t="s">
+        <v>93</v>
+      </c>
+      <c r="F54" t="s">
+        <v>117</v>
+      </c>
+      <c r="G54" t="s">
+        <v>170</v>
+      </c>
+      <c r="H54" t="s">
+        <v>182</v>
+      </c>
+      <c r="I54">
+        <v>0</v>
+      </c>
+      <c r="J54" t="s">
+        <v>185</v>
+      </c>
+      <c r="K54" t="s">
+        <v>187</v>
+      </c>
+      <c r="L54">
+        <v>1549</v>
+      </c>
+      <c r="M54" t="s">
+        <v>191</v>
+      </c>
+      <c r="O54" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16">
+      <c r="A55">
+        <v>53</v>
+      </c>
+      <c r="B55">
+        <v>100483</v>
+      </c>
+      <c r="C55">
+        <v>360852</v>
+      </c>
+      <c r="D55" t="s">
+        <v>39</v>
+      </c>
+      <c r="E55" t="s">
+        <v>94</v>
+      </c>
+      <c r="F55" t="s">
+        <v>100</v>
+      </c>
+      <c r="G55" t="s">
+        <v>171</v>
+      </c>
+      <c r="H55" t="s">
+        <v>176</v>
+      </c>
+      <c r="I55">
+        <v>0</v>
+      </c>
+      <c r="J55" t="s">
+        <v>185</v>
+      </c>
+      <c r="K55" t="s">
+        <v>187</v>
+      </c>
+      <c r="L55">
+        <v>649</v>
+      </c>
+      <c r="M55">
+        <v>11</v>
+      </c>
+      <c r="N55" t="s">
+        <v>226</v>
+      </c>
+      <c r="O55" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16">
+      <c r="A56">
+        <v>54</v>
+      </c>
+      <c r="B56">
+        <v>100515</v>
+      </c>
+      <c r="C56">
+        <v>361056</v>
+      </c>
+      <c r="D56" t="s">
+        <v>40</v>
+      </c>
+      <c r="E56" t="s">
+        <v>95</v>
+      </c>
+      <c r="F56" t="s">
+        <v>100</v>
+      </c>
+      <c r="G56" t="s">
+        <v>172</v>
+      </c>
+      <c r="H56" t="s">
+        <v>178</v>
+      </c>
+      <c r="I56">
+        <v>0</v>
+      </c>
+      <c r="J56" t="s">
+        <v>185</v>
+      </c>
+      <c r="K56" t="s">
+        <v>187</v>
+      </c>
+      <c r="L56">
+        <v>649</v>
+      </c>
+      <c r="M56">
+        <v>11</v>
+      </c>
+      <c r="N56" t="s">
+        <v>227</v>
+      </c>
+      <c r="O56" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16">
+      <c r="A57">
+        <v>55</v>
+      </c>
+      <c r="B57">
+        <v>98943</v>
+      </c>
+      <c r="C57">
+        <v>37106</v>
+      </c>
+      <c r="D57">
+        <v>34985</v>
+      </c>
+      <c r="E57" t="s">
+        <v>96</v>
+      </c>
+      <c r="F57" t="s">
+        <v>101</v>
+      </c>
+      <c r="G57" t="s">
+        <v>173</v>
+      </c>
+      <c r="H57" t="s">
+        <v>176</v>
+      </c>
+      <c r="I57">
+        <v>0</v>
+      </c>
+      <c r="J57" t="s">
+        <v>185</v>
+      </c>
+      <c r="K57" t="s">
+        <v>188</v>
+      </c>
+      <c r="L57">
+        <v>399</v>
+      </c>
+      <c r="M57" t="s">
+        <v>191</v>
+      </c>
+      <c r="O57" t="s">
+        <v>230</v>
+      </c>
+      <c r="P57">
+        <v>96274</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16">
+      <c r="A58">
+        <v>56</v>
+      </c>
+      <c r="B58">
         <v>100497</v>
       </c>
-      <c r="C39">
+      <c r="C58">
         <v>179725</v>
       </c>
-      <c r="D39">
+      <c r="D58">
         <v>77232</v>
       </c>
-      <c r="E39" t="s">
-        <v>72</v>
-      </c>
-      <c r="F39" t="s">
-        <v>75</v>
-      </c>
-      <c r="G39" t="s">
-        <v>128</v>
-      </c>
-      <c r="H39" t="s">
-        <v>130</v>
-      </c>
-      <c r="I39">
-        <v>0</v>
-      </c>
-      <c r="J39" t="s">
-        <v>136</v>
-      </c>
-      <c r="K39" t="s">
-        <v>138</v>
-      </c>
-      <c r="L39">
+      <c r="E58" t="s">
+        <v>97</v>
+      </c>
+      <c r="F58" t="s">
+        <v>105</v>
+      </c>
+      <c r="G58" t="s">
+        <v>174</v>
+      </c>
+      <c r="H58" t="s">
+        <v>176</v>
+      </c>
+      <c r="I58">
+        <v>0</v>
+      </c>
+      <c r="J58" t="s">
+        <v>185</v>
+      </c>
+      <c r="K58" t="s">
+        <v>188</v>
+      </c>
+      <c r="L58">
         <v>499</v>
       </c>
-      <c r="M39">
+      <c r="M58">
         <v>11</v>
       </c>
-      <c r="N39" t="s">
-        <v>165</v>
-      </c>
-      <c r="O39" t="s">
-        <v>167</v>
-      </c>
-      <c r="P39">
+      <c r="N58" t="s">
+        <v>228</v>
+      </c>
+      <c r="O58" t="s">
+        <v>231</v>
+      </c>
+      <c r="P58">
         <v>4540</v>
       </c>
     </row>
-    <row r="40" spans="1:16">
-      <c r="A40" t="s">
+    <row r="59" spans="1:16">
+      <c r="A59" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Link Track daily mart rows to version records
</commit_message>
<xml_diff>
--- a/backend/data/cargos_recurrentes/cargos_recurrentes.xlsx
+++ b/backend/data/cargos_recurrentes/cargos_recurrentes.xlsx
@@ -67,7 +67,7 @@
     <t>Unnamed: 16</t>
   </si>
   <si>
-    <t>Reporte generado: 02-05-2026 03:43 p. m.</t>
+    <t>Reporte generado: 02-05-2026 05:54 p. m.</t>
   </si>
   <si>
     <t>Folio</t>
@@ -79,6 +79,21 @@
     <t>PIN</t>
   </si>
   <si>
+    <t>03156</t>
+  </si>
+  <si>
+    <t>02589</t>
+  </si>
+  <si>
+    <t>03053</t>
+  </si>
+  <si>
+    <t>03183</t>
+  </si>
+  <si>
+    <t>09543</t>
+  </si>
+  <si>
     <t>02210</t>
   </si>
   <si>
@@ -88,6 +103,9 @@
     <t>03168</t>
   </si>
   <si>
+    <t>03219</t>
+  </si>
+  <si>
     <t>09964</t>
   </si>
   <si>
@@ -106,30 +124,12 @@
     <t>02795</t>
   </si>
   <si>
-    <t>03156</t>
-  </si>
-  <si>
-    <t>02589</t>
-  </si>
-  <si>
-    <t>03053</t>
-  </si>
-  <si>
-    <t>03183</t>
-  </si>
-  <si>
     <t>03034</t>
   </si>
   <si>
     <t>03191</t>
   </si>
   <si>
-    <t>03219</t>
-  </si>
-  <si>
-    <t>09543</t>
-  </si>
-  <si>
     <t>03005</t>
   </si>
   <si>
@@ -142,6 +142,72 @@
     <t>Nombre</t>
   </si>
   <si>
+    <t>CESAR DANIEL  PEREYRA  CONTRERAS</t>
+  </si>
+  <si>
+    <t>JOSE MANUEL OSUNA PEÑA</t>
+  </si>
+  <si>
+    <t>DANIA FERNANDA MORENO BELLO</t>
+  </si>
+  <si>
+    <t>MARLENE  GARCIA AGUILAR</t>
+  </si>
+  <si>
+    <t>NATALIA PADILLA RIVAS</t>
+  </si>
+  <si>
+    <t>ERIKA ADRIANA BERMUDEZ TALAVERA</t>
+  </si>
+  <si>
+    <t>ISRAEL CRESPO RIOS</t>
+  </si>
+  <si>
+    <t>JULIO CESAR VERDE  MANJARRES</t>
+  </si>
+  <si>
+    <t>JESUS ANTONIO ABRIL CAMPOS</t>
+  </si>
+  <si>
+    <t>ALMA ANGELICA  PEREZ  MIRANDA</t>
+  </si>
+  <si>
+    <t>MARA FERNANDA LUNA MENDOZA</t>
+  </si>
+  <si>
+    <t>NOEMI  RAMOS  DE LEON</t>
+  </si>
+  <si>
+    <t>DENIS LILIANA AMEZCUA CRUZ</t>
+  </si>
+  <si>
+    <t>LUIS DAVID ROSAS  ALONSO</t>
+  </si>
+  <si>
+    <t>ALEJANDRO MAGALLAN  LOPEZ</t>
+  </si>
+  <si>
+    <t>NIRVANA FERNANDA  SALADO  SANCHEZ</t>
+  </si>
+  <si>
+    <t>ANA LUISA  HERNANDEZ  BELTRAN</t>
+  </si>
+  <si>
+    <t>ELOINA  REYNOSO  TERRONES</t>
+  </si>
+  <si>
+    <t>ANA FABIOLA FLORES CARMONA</t>
+  </si>
+  <si>
+    <t>GUILLERMO GERARDO VAZQUEZ GARCIA</t>
+  </si>
+  <si>
+    <t>JUAN  FLORES  FELIX</t>
+  </si>
+  <si>
+    <t>FELIPE ALFONSO GUERRERO INZUNZA</t>
+  </si>
+  <si>
     <t>BALTAZAR VILLASEÑOR  CRUZ</t>
   </si>
   <si>
@@ -154,12 +220,36 @@
     <t>DEMIAN CORONADO LOPEZ</t>
   </si>
   <si>
-    <t>FELIPE ALFONSO GUERRERO INZUNZA</t>
+    <t>YOSHIO JESUS  RINCON  MIRANDA</t>
+  </si>
+  <si>
+    <t>LETICIA RUBIO VALENZUELA</t>
+  </si>
+  <si>
+    <t>BRISEIDA ISABEL ENRIQUEZ ZEPEDA</t>
+  </si>
+  <si>
+    <t>DULCE NOHEMI SOTO MORENO</t>
+  </si>
+  <si>
+    <t>JUAN JOSE  PACHECO  FLORES</t>
+  </si>
+  <si>
+    <t>CHRISTIAN PRISCILA CARDONA BANDA</t>
+  </si>
+  <si>
+    <t>ALAN IGNACIO  CORTES HERNANDEZ</t>
+  </si>
+  <si>
+    <t>SUSAN ELIZABETH SOTO PIÑA</t>
   </si>
   <si>
     <t>LILIAN RUVALCABA FIGUEROA</t>
   </si>
   <si>
+    <t>LARISSA DENISSE LOPEZ BURGOS</t>
+  </si>
+  <si>
     <t>GUADALUPE  CASTRO ROSAS</t>
   </si>
   <si>
@@ -181,54 +271,12 @@
     <t>EDUARDO  GONZALES FLORES</t>
   </si>
   <si>
-    <t>LARISSA DENISSE LOPEZ BURGOS</t>
-  </si>
-  <si>
-    <t>JOSE MANUEL OSUNA PEÑA</t>
-  </si>
-  <si>
-    <t>DANIA FERNANDA MORENO BELLO</t>
-  </si>
-  <si>
-    <t>MARLENE  GARCIA AGUILAR</t>
-  </si>
-  <si>
-    <t>NATALIA PADILLA RIVAS</t>
-  </si>
-  <si>
-    <t>CESAR DANIEL  PEREYRA  CONTRERAS</t>
-  </si>
-  <si>
-    <t>ERIKA ADRIANA BERMUDEZ TALAVERA</t>
-  </si>
-  <si>
-    <t>ISRAEL CRESPO RIOS</t>
-  </si>
-  <si>
-    <t>JULIO CESAR VERDE  MANJARRES</t>
-  </si>
-  <si>
-    <t>JESUS ANTONIO ABRIL CAMPOS</t>
-  </si>
-  <si>
-    <t>MARA FERNANDA LUNA MENDOZA</t>
-  </si>
-  <si>
-    <t>NOEMI  RAMOS  DE LEON</t>
-  </si>
-  <si>
-    <t>DENIS LILIANA AMEZCUA CRUZ</t>
-  </si>
-  <si>
-    <t>LUIS DAVID ROSAS  ALONSO</t>
-  </si>
-  <si>
-    <t>ALMA ANGELICA  PEREZ  MIRANDA</t>
-  </si>
-  <si>
     <t>ANGELICA DEYANIRA SERRANO VALDEZ</t>
   </si>
   <si>
+    <t>MONICA DANIELA  ORDUÑO PEREZ</t>
+  </si>
+  <si>
     <t>ELISA ELENA PAREDES HERNANDEZ</t>
   </si>
   <si>
@@ -247,88 +295,70 @@
     <t>HILARY MONROY MORENO</t>
   </si>
   <si>
-    <t>MONICA DANIELA  ORDUÑO PEREZ</t>
-  </si>
-  <si>
-    <t>JUAN JOSE  PACHECO  FLORES</t>
-  </si>
-  <si>
-    <t>DULCE NOHEMI SOTO MORENO</t>
-  </si>
-  <si>
-    <t>SUSAN ELIZABETH SOTO PIÑA</t>
-  </si>
-  <si>
-    <t>CHRISTIAN PRISCILA CARDONA BANDA</t>
-  </si>
-  <si>
-    <t>ALAN IGNACIO  CORTES HERNANDEZ</t>
-  </si>
-  <si>
-    <t>YOSHIO JESUS  RINCON  MIRANDA</t>
-  </si>
-  <si>
-    <t>LETICIA RUBIO VALENZUELA</t>
-  </si>
-  <si>
-    <t>BRISEIDA ISABEL ENRIQUEZ ZEPEDA</t>
-  </si>
-  <si>
-    <t>ANA LUISA  HERNANDEZ  BELTRAN</t>
-  </si>
-  <si>
-    <t>ANA FABIOLA FLORES CARMONA</t>
-  </si>
-  <si>
-    <t>GUILLERMO GERARDO VAZQUEZ GARCIA</t>
-  </si>
-  <si>
-    <t>JUAN  FLORES  FELIX</t>
-  </si>
-  <si>
-    <t>ALEJANDRO MAGALLAN  LOPEZ</t>
-  </si>
-  <si>
-    <t>NIRVANA FERNANDA  SALADO  SANCHEZ</t>
-  </si>
-  <si>
-    <t>ELOINA  REYNOSO  TERRONES</t>
-  </si>
-  <si>
     <t>TANIA ELIZABETH VILLAREAL PEREDA</t>
   </si>
   <si>
     <t>ELIUD RAMIREZ BELMARES</t>
   </si>
   <si>
+    <t>JUAN FRANCISCO PITONES NORIEGA</t>
+  </si>
+  <si>
     <t>GILBERTO  BARRIOS HERNANDEZ</t>
   </si>
   <si>
-    <t>JUAN FRANCISCO PITONES NORIEGA</t>
-  </si>
-  <si>
     <t>EBER  MAGDIEL  CASTILLEJA  BARROSO</t>
   </si>
   <si>
     <t>Sucursal</t>
   </si>
   <si>
+    <t>VILLA VERDE</t>
+  </si>
+  <si>
+    <t>PASEO 2000</t>
+  </si>
+  <si>
+    <t>TEC MXL</t>
+  </si>
+  <si>
+    <t>CARROUSEL TJ</t>
+  </si>
+  <si>
+    <t>MISION ENS</t>
+  </si>
+  <si>
+    <t>SAN LUIS</t>
+  </si>
+  <si>
+    <t>SANTA FE</t>
+  </si>
+  <si>
+    <t>SEND CUL</t>
+  </si>
+  <si>
+    <t>AZAHARES CUL</t>
+  </si>
+  <si>
+    <t>PABELLON RTO</t>
+  </si>
+  <si>
+    <t>SEND MXL</t>
+  </si>
+  <si>
     <t>METEPEC</t>
   </si>
   <si>
     <t>SALTILLO VILLALTA</t>
   </si>
   <si>
-    <t>SEND MXL</t>
-  </si>
-  <si>
-    <t>TEC MXL</t>
-  </si>
-  <si>
-    <t>SEND CUL</t>
-  </si>
-  <si>
-    <t>MISION ENS</t>
+    <t>INDEPENDENCIA</t>
+  </si>
+  <si>
+    <t>PAPALOTE TJ</t>
+  </si>
+  <si>
+    <t>STA CATARINA</t>
   </si>
   <si>
     <t>SEND SALTILLO</t>
@@ -337,42 +367,78 @@
     <t>IXTAPALUCA</t>
   </si>
   <si>
-    <t>PASEO 2000</t>
-  </si>
-  <si>
-    <t>VILLA VERDE</t>
-  </si>
-  <si>
-    <t>CARROUSEL TJ</t>
-  </si>
-  <si>
-    <t>SAN LUIS</t>
-  </si>
-  <si>
-    <t>SANTA FE</t>
-  </si>
-  <si>
-    <t>STA CATARINA</t>
-  </si>
-  <si>
-    <t>INDEPENDENCIA</t>
-  </si>
-  <si>
-    <t>PAPALOTE TJ</t>
-  </si>
-  <si>
-    <t>AZAHARES CUL</t>
-  </si>
-  <si>
-    <t>PABELLON RTO</t>
-  </si>
-  <si>
     <t>INSURGENTES</t>
   </si>
   <si>
     <t>Fecha Inicio</t>
   </si>
   <si>
+    <t>10-04-2026 17:32:18</t>
+  </si>
+  <si>
+    <t>01-05-2026 9:28:55</t>
+  </si>
+  <si>
+    <t>01-05-2026 12:44:57</t>
+  </si>
+  <si>
+    <t>01-05-2026 17:35:18</t>
+  </si>
+  <si>
+    <t>02-05-2026 13:06:35</t>
+  </si>
+  <si>
+    <t>21-04-2026 13:14:32</t>
+  </si>
+  <si>
+    <t>02-04-2026 11:27:04</t>
+  </si>
+  <si>
+    <t>03-04-2026 10:04:26</t>
+  </si>
+  <si>
+    <t>06-04-2026 5:30:30</t>
+  </si>
+  <si>
+    <t>20-04-2026 20:14:31</t>
+  </si>
+  <si>
+    <t>01-05-2026 10:38:33</t>
+  </si>
+  <si>
+    <t>01-05-2026 11:15:25</t>
+  </si>
+  <si>
+    <t>01-05-2026 19:13:51</t>
+  </si>
+  <si>
+    <t>02-05-2026 13:24:03</t>
+  </si>
+  <si>
+    <t>02-04-2026 7:19:31</t>
+  </si>
+  <si>
+    <t>02-04-2026 11:24:30</t>
+  </si>
+  <si>
+    <t>01-05-2026 10:01:13</t>
+  </si>
+  <si>
+    <t>10-04-2026 15:14:18</t>
+  </si>
+  <si>
+    <t>01-05-2026 11:54:51</t>
+  </si>
+  <si>
+    <t>01-05-2026 16:31:24</t>
+  </si>
+  <si>
+    <t>01-05-2026 20:54:12</t>
+  </si>
+  <si>
+    <t>14-04-2026 12:19:40</t>
+  </si>
+  <si>
     <t>01-05-2026 11:51:52</t>
   </si>
   <si>
@@ -385,12 +451,36 @@
     <t>01-05-2026 18:12:55</t>
   </si>
   <si>
-    <t>14-04-2026 12:19:40</t>
+    <t>03-04-2026 17:05:50</t>
+  </si>
+  <si>
+    <t>07-04-2026 17:54:05</t>
+  </si>
+  <si>
+    <t>20-04-2026 21:29:56</t>
+  </si>
+  <si>
+    <t>24-03-2026 20:48:40</t>
+  </si>
+  <si>
+    <t>28-04-2026 13:00:52</t>
+  </si>
+  <si>
+    <t>01-05-2026 16:18:47</t>
+  </si>
+  <si>
+    <t>02-05-2026 7:36:52</t>
+  </si>
+  <si>
+    <t>26-03-2026 13:42:06</t>
   </si>
   <si>
     <t>21-04-2026 13:16:43</t>
   </si>
   <si>
+    <t>31-03-2026 20:18:54</t>
+  </si>
+  <si>
     <t>24-04-2026 15:34:48</t>
   </si>
   <si>
@@ -412,54 +502,12 @@
     <t>02-05-2026 13:13:57</t>
   </si>
   <si>
-    <t>31-03-2026 20:18:54</t>
-  </si>
-  <si>
-    <t>01-05-2026 9:28:55</t>
-  </si>
-  <si>
-    <t>01-05-2026 12:44:57</t>
-  </si>
-  <si>
-    <t>01-05-2026 17:35:18</t>
-  </si>
-  <si>
-    <t>02-05-2026 13:06:35</t>
-  </si>
-  <si>
-    <t>10-04-2026 17:32:18</t>
-  </si>
-  <si>
-    <t>21-04-2026 13:14:32</t>
-  </si>
-  <si>
-    <t>02-04-2026 11:27:04</t>
-  </si>
-  <si>
-    <t>03-04-2026 10:04:26</t>
-  </si>
-  <si>
-    <t>06-04-2026 5:30:30</t>
-  </si>
-  <si>
-    <t>01-05-2026 10:38:33</t>
-  </si>
-  <si>
-    <t>01-05-2026 11:15:25</t>
-  </si>
-  <si>
-    <t>01-05-2026 19:13:51</t>
-  </si>
-  <si>
-    <t>02-05-2026 13:24:03</t>
-  </si>
-  <si>
-    <t>20-04-2026 20:14:31</t>
-  </si>
-  <si>
     <t>04-03-2026 15:59:55</t>
   </si>
   <si>
+    <t>11-04-2026 10:17:07</t>
+  </si>
+  <si>
     <t>27-04-2026 8:15:35</t>
   </si>
   <si>
@@ -478,66 +526,18 @@
     <t>01-05-2026 20:07:30</t>
   </si>
   <si>
-    <t>11-04-2026 10:17:07</t>
-  </si>
-  <si>
-    <t>28-04-2026 13:00:52</t>
-  </si>
-  <si>
-    <t>24-03-2026 20:48:40</t>
-  </si>
-  <si>
-    <t>26-03-2026 13:42:06</t>
-  </si>
-  <si>
-    <t>01-05-2026 16:18:47</t>
-  </si>
-  <si>
-    <t>02-05-2026 7:36:52</t>
-  </si>
-  <si>
-    <t>03-04-2026 17:05:50</t>
-  </si>
-  <si>
-    <t>07-04-2026 17:54:05</t>
-  </si>
-  <si>
-    <t>20-04-2026 21:29:56</t>
-  </si>
-  <si>
-    <t>01-05-2026 10:01:13</t>
-  </si>
-  <si>
-    <t>01-05-2026 11:54:51</t>
-  </si>
-  <si>
-    <t>01-05-2026 16:31:24</t>
-  </si>
-  <si>
-    <t>01-05-2026 20:54:12</t>
-  </si>
-  <si>
-    <t>02-04-2026 7:19:31</t>
-  </si>
-  <si>
-    <t>02-04-2026 11:24:30</t>
-  </si>
-  <si>
-    <t>10-04-2026 15:14:18</t>
-  </si>
-  <si>
     <t>01-05-2026 7:38:40</t>
   </si>
   <si>
     <t>01-05-2026 8:37:34</t>
   </si>
   <si>
+    <t>08-04-2026 20:42:26</t>
+  </si>
+  <si>
     <t>02-05-2026 7:46:19</t>
   </si>
   <si>
-    <t>08-04-2026 20:42:26</t>
-  </si>
-  <si>
     <t>01-05-2026 15:17:21</t>
   </si>
   <si>
@@ -547,21 +547,21 @@
     <t>01-06-2026 23:59:59</t>
   </si>
   <si>
+    <t>02-06-2026 23:59:59</t>
+  </si>
+  <si>
+    <t>04-06-2026 23:59:59</t>
+  </si>
+  <si>
     <t>30-05-2026 23:59:59</t>
   </si>
   <si>
-    <t>02-06-2026 23:59:59</t>
-  </si>
-  <si>
-    <t>04-06-2026 23:59:59</t>
+    <t>10-05-2026 23:59:59</t>
   </si>
   <si>
     <t>03-05-2026 23:59:59</t>
   </si>
   <si>
-    <t>10-05-2026 23:59:59</t>
-  </si>
-  <si>
     <t>01-08-2026 23:59:59</t>
   </si>
   <si>
@@ -577,12 +577,12 @@
     <t>Estatus</t>
   </si>
   <si>
+    <t>RENOVACIÓN</t>
+  </si>
+  <si>
     <t>NUEVO</t>
   </si>
   <si>
-    <t>RENOVACIÓN</t>
-  </si>
-  <si>
     <t>Importe</t>
   </si>
   <si>
@@ -595,15 +595,81 @@
     <t>Fecha Fin Contrato</t>
   </si>
   <si>
+    <t>26-04-2027 9:28:55</t>
+  </si>
+  <si>
+    <t>26-04-2027 12:44:57</t>
+  </si>
+  <si>
+    <t>27-04-2027 13:06:35</t>
+  </si>
+  <si>
+    <t>16-04-2027 13:14:32</t>
+  </si>
+  <si>
+    <t>28-03-2027 11:27:04</t>
+  </si>
+  <si>
+    <t>30-09-2026 10:04:26</t>
+  </si>
+  <si>
+    <t>26-04-2027 11:15:25</t>
+  </si>
+  <si>
+    <t>27-04-2027 13:24:03</t>
+  </si>
+  <si>
+    <t>29-09-2026 7:19:31</t>
+  </si>
+  <si>
+    <t>28-03-2027 11:24:30</t>
+  </si>
+  <si>
+    <t>26-04-2027 10:01:13</t>
+  </si>
+  <si>
+    <t>26-04-2027 11:54:51</t>
+  </si>
+  <si>
+    <t>26-04-2027 16:31:24</t>
+  </si>
+  <si>
+    <t>28-10-2026 20:54:12</t>
+  </si>
+  <si>
     <t>26-04-2027 12:28:55</t>
   </si>
   <si>
     <t>28-10-2026 17:19:17</t>
   </si>
   <si>
+    <t>30-09-2026 17:05:50</t>
+  </si>
+  <si>
+    <t>02-04-2027 17:54:05</t>
+  </si>
+  <si>
+    <t>15-04-2027 21:29:56</t>
+  </si>
+  <si>
+    <t>19-03-2027 20:48:40</t>
+  </si>
+  <si>
+    <t>26-04-2027 16:18:47</t>
+  </si>
+  <si>
+    <t>27-04-2027 7:36:52</t>
+  </si>
+  <si>
+    <t>21-03-2027 13:42:06</t>
+  </si>
+  <si>
     <t>16-04-2027 13:16:43</t>
   </si>
   <si>
+    <t>26-03-2027 20:18:54</t>
+  </si>
+  <si>
     <t>21-10-2026 15:34:48</t>
   </si>
   <si>
@@ -619,33 +685,6 @@
     <t>26-04-2027 18:32:13</t>
   </si>
   <si>
-    <t>26-03-2027 20:18:54</t>
-  </si>
-  <si>
-    <t>26-04-2027 9:28:55</t>
-  </si>
-  <si>
-    <t>26-04-2027 12:44:57</t>
-  </si>
-  <si>
-    <t>27-04-2027 13:06:35</t>
-  </si>
-  <si>
-    <t>16-04-2027 13:14:32</t>
-  </si>
-  <si>
-    <t>28-03-2027 11:27:04</t>
-  </si>
-  <si>
-    <t>30-09-2026 10:04:26</t>
-  </si>
-  <si>
-    <t>26-04-2027 11:15:25</t>
-  </si>
-  <si>
-    <t>27-04-2027 13:24:03</t>
-  </si>
-  <si>
     <t>27-02-2027 15:59:55</t>
   </si>
   <si>
@@ -653,45 +692,6 @@
   </si>
   <si>
     <t>26-04-2027 20:01:10</t>
-  </si>
-  <si>
-    <t>19-03-2027 20:48:40</t>
-  </si>
-  <si>
-    <t>21-03-2027 13:42:06</t>
-  </si>
-  <si>
-    <t>26-04-2027 16:18:47</t>
-  </si>
-  <si>
-    <t>27-04-2027 7:36:52</t>
-  </si>
-  <si>
-    <t>30-09-2026 17:05:50</t>
-  </si>
-  <si>
-    <t>02-04-2027 17:54:05</t>
-  </si>
-  <si>
-    <t>15-04-2027 21:29:56</t>
-  </si>
-  <si>
-    <t>26-04-2027 10:01:13</t>
-  </si>
-  <si>
-    <t>26-04-2027 11:54:51</t>
-  </si>
-  <si>
-    <t>26-04-2027 16:31:24</t>
-  </si>
-  <si>
-    <t>28-10-2026 20:54:12</t>
-  </si>
-  <si>
-    <t>29-09-2026 7:19:31</t>
-  </si>
-  <si>
-    <t>28-03-2027 11:24:30</t>
   </si>
   <si>
     <t>26-04-2027 8:37:34</t>
@@ -1184,13 +1184,13 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>100493</v>
+        <v>99056</v>
       </c>
       <c r="C3">
-        <v>360045</v>
-      </c>
-      <c r="D3" t="s">
-        <v>21</v>
+        <v>76774</v>
+      </c>
+      <c r="D3">
+        <v>74576</v>
       </c>
       <c r="E3" t="s">
         <v>42</v>
@@ -1214,13 +1214,16 @@
         <v>187</v>
       </c>
       <c r="L3">
-        <v>799</v>
+        <v>399</v>
       </c>
       <c r="M3" t="s">
         <v>191</v>
       </c>
       <c r="O3" t="s">
         <v>230</v>
+      </c>
+      <c r="P3">
+        <v>24188</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -1228,13 +1231,13 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>100495</v>
+        <v>100485</v>
       </c>
       <c r="C4">
-        <v>349026</v>
+        <v>283428</v>
       </c>
       <c r="D4">
-        <v>91191</v>
+        <v>80929</v>
       </c>
       <c r="E4" t="s">
         <v>43</v>
@@ -1258,7 +1261,7 @@
         <v>187</v>
       </c>
       <c r="L4">
-        <v>649</v>
+        <v>699</v>
       </c>
       <c r="M4">
         <v>11</v>
@@ -1268,6 +1271,9 @@
       </c>
       <c r="O4" t="s">
         <v>231</v>
+      </c>
+      <c r="P4">
+        <v>60636</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -1275,13 +1281,13 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>100502</v>
+        <v>100496</v>
       </c>
       <c r="C5">
-        <v>205459</v>
-      </c>
-      <c r="D5" t="s">
-        <v>22</v>
+        <v>241908</v>
+      </c>
+      <c r="D5">
+        <v>39413</v>
       </c>
       <c r="E5" t="s">
         <v>44</v>
@@ -1293,7 +1299,7 @@
         <v>121</v>
       </c>
       <c r="H5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -1302,13 +1308,13 @@
         <v>185</v>
       </c>
       <c r="K5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L5">
-        <v>399</v>
+        <v>699</v>
       </c>
       <c r="M5">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="N5" t="s">
         <v>194</v>
@@ -1317,7 +1323,7 @@
         <v>231</v>
       </c>
       <c r="P5">
-        <v>38806</v>
+        <v>54257</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -1325,19 +1331,19 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>100504</v>
+        <v>100503</v>
       </c>
       <c r="C6">
-        <v>361003</v>
+        <v>360991</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E6" t="s">
         <v>45</v>
       </c>
       <c r="F6" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G6" t="s">
         <v>122</v>
@@ -1352,7 +1358,7 @@
         <v>185</v>
       </c>
       <c r="K6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L6">
         <v>649</v>
@@ -1369,25 +1375,25 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>99332</v>
+        <v>100521</v>
       </c>
       <c r="C7">
-        <v>257916</v>
+        <v>266562</v>
       </c>
       <c r="D7">
-        <v>55420</v>
+        <v>64066</v>
       </c>
       <c r="E7" t="s">
         <v>46</v>
       </c>
       <c r="F7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G7" t="s">
         <v>123</v>
       </c>
       <c r="H7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -1399,16 +1405,16 @@
         <v>188</v>
       </c>
       <c r="L7">
-        <v>399</v>
-      </c>
-      <c r="M7" t="s">
-        <v>191</v>
+        <v>499</v>
+      </c>
+      <c r="M7">
+        <v>11</v>
+      </c>
+      <c r="N7" t="s">
+        <v>195</v>
       </c>
       <c r="O7" t="s">
-        <v>230</v>
-      </c>
-      <c r="P7">
-        <v>73999</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -1416,25 +1422,25 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>99890</v>
+        <v>99889</v>
       </c>
       <c r="C8">
-        <v>34927</v>
+        <v>17586</v>
       </c>
       <c r="D8">
-        <v>32841</v>
+        <v>16499</v>
       </c>
       <c r="E8" t="s">
         <v>47</v>
       </c>
       <c r="F8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G8" t="s">
         <v>124</v>
       </c>
       <c r="H8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -1443,7 +1449,7 @@
         <v>185</v>
       </c>
       <c r="K8" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L8">
         <v>499</v>
@@ -1452,13 +1458,13 @@
         <v>11</v>
       </c>
       <c r="N8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="O8" t="s">
         <v>231</v>
       </c>
       <c r="P8">
-        <v>95584</v>
+        <v>95586</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -1466,25 +1472,25 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>100107</v>
+        <v>98466</v>
       </c>
       <c r="C9">
-        <v>312465</v>
+        <v>205081</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E9" t="s">
         <v>48</v>
       </c>
       <c r="F9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G9" t="s">
         <v>125</v>
       </c>
       <c r="H9" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -1493,22 +1499,22 @@
         <v>185</v>
       </c>
       <c r="K9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L9">
-        <v>549</v>
+        <v>499</v>
       </c>
       <c r="M9">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="N9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O9" t="s">
         <v>231</v>
       </c>
       <c r="P9">
-        <v>77036</v>
+        <v>76809</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -1516,25 +1522,25 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>100488</v>
+        <v>98517</v>
       </c>
       <c r="C10">
-        <v>360887</v>
-      </c>
-      <c r="D10" t="s">
-        <v>25</v>
+        <v>232630</v>
+      </c>
+      <c r="D10">
+        <v>30135</v>
       </c>
       <c r="E10" t="s">
         <v>49</v>
       </c>
       <c r="F10" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G10" t="s">
         <v>126</v>
       </c>
       <c r="H10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -1546,16 +1552,19 @@
         <v>187</v>
       </c>
       <c r="L10">
-        <v>549</v>
+        <v>449</v>
       </c>
       <c r="M10">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O10" t="s">
         <v>231</v>
+      </c>
+      <c r="P10">
+        <v>49260</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -1563,19 +1572,19 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>100490</v>
+        <v>98583</v>
       </c>
       <c r="C11">
-        <v>360892</v>
-      </c>
-      <c r="D11" t="s">
-        <v>26</v>
+        <v>114721</v>
+      </c>
+      <c r="D11">
+        <v>12446</v>
       </c>
       <c r="E11" t="s">
         <v>50</v>
       </c>
       <c r="F11" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G11" t="s">
         <v>127</v>
@@ -1593,13 +1602,16 @@
         <v>187</v>
       </c>
       <c r="L11">
-        <v>649</v>
+        <v>399</v>
       </c>
       <c r="M11" t="s">
         <v>191</v>
       </c>
       <c r="O11" t="s">
         <v>230</v>
+      </c>
+      <c r="P11">
+        <v>11835</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -1607,19 +1619,19 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>100492</v>
+        <v>99840</v>
       </c>
       <c r="C12">
-        <v>360904</v>
-      </c>
-      <c r="D12" t="s">
-        <v>27</v>
+        <v>178067</v>
+      </c>
+      <c r="D12">
+        <v>75574</v>
       </c>
       <c r="E12" t="s">
         <v>51</v>
       </c>
       <c r="F12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G12" t="s">
         <v>128</v>
@@ -1637,16 +1649,16 @@
         <v>187</v>
       </c>
       <c r="L12">
-        <v>549</v>
-      </c>
-      <c r="M12">
-        <v>11</v>
-      </c>
-      <c r="N12" t="s">
-        <v>198</v>
+        <v>449</v>
+      </c>
+      <c r="M12" t="s">
+        <v>191</v>
       </c>
       <c r="O12" t="s">
-        <v>231</v>
+        <v>230</v>
+      </c>
+      <c r="P12">
+        <v>74406</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -1654,19 +1666,19 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>100505</v>
+        <v>100489</v>
       </c>
       <c r="C13">
-        <v>360757</v>
+        <v>360888</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="E13" t="s">
         <v>52</v>
       </c>
       <c r="F13" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G13" t="s">
         <v>129</v>
@@ -1681,19 +1693,16 @@
         <v>185</v>
       </c>
       <c r="K13" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L13">
-        <v>549</v>
-      </c>
-      <c r="M13">
-        <v>11</v>
-      </c>
-      <c r="N13" t="s">
-        <v>199</v>
+        <v>649</v>
+      </c>
+      <c r="M13" t="s">
+        <v>191</v>
       </c>
       <c r="O13" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -1701,25 +1710,25 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>100507</v>
+        <v>100491</v>
       </c>
       <c r="C14">
-        <v>353643</v>
+        <v>56971</v>
       </c>
       <c r="D14">
-        <v>95807</v>
+        <v>54822</v>
       </c>
       <c r="E14" t="s">
         <v>53</v>
       </c>
       <c r="F14" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="G14" t="s">
         <v>130</v>
       </c>
       <c r="H14" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="I14">
         <v>0</v>
@@ -1731,16 +1740,19 @@
         <v>187</v>
       </c>
       <c r="L14">
-        <v>649</v>
+        <v>449</v>
       </c>
       <c r="M14">
         <v>11</v>
       </c>
       <c r="N14" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="O14" t="s">
         <v>231</v>
+      </c>
+      <c r="P14">
+        <v>68495</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -1748,25 +1760,25 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>100522</v>
+        <v>100508</v>
       </c>
       <c r="C15">
-        <v>360630</v>
+        <v>361018</v>
       </c>
       <c r="D15" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E15" t="s">
         <v>54</v>
       </c>
       <c r="F15" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G15" t="s">
         <v>131</v>
       </c>
       <c r="H15" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="I15">
         <v>0</v>
@@ -1775,10 +1787,10 @@
         <v>185</v>
       </c>
       <c r="K15" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L15">
-        <v>549</v>
+        <v>649</v>
       </c>
       <c r="M15" t="s">
         <v>191</v>
@@ -1792,25 +1804,25 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>98369</v>
+        <v>100523</v>
       </c>
       <c r="C16">
-        <v>56575</v>
+        <v>177956</v>
       </c>
       <c r="D16">
-        <v>54426</v>
+        <v>75463</v>
       </c>
       <c r="E16" t="s">
         <v>55</v>
       </c>
       <c r="F16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G16" t="s">
         <v>132</v>
       </c>
       <c r="H16" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I16">
         <v>0</v>
@@ -1819,7 +1831,7 @@
         <v>185</v>
       </c>
       <c r="K16" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L16">
         <v>499</v>
@@ -1828,13 +1840,13 @@
         <v>11</v>
       </c>
       <c r="N16" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O16" t="s">
         <v>231</v>
       </c>
       <c r="P16">
-        <v>91270</v>
+        <v>4701</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -1842,19 +1854,19 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>100485</v>
+        <v>98454</v>
       </c>
       <c r="C17">
-        <v>283428</v>
+        <v>65078</v>
       </c>
       <c r="D17">
-        <v>80929</v>
+        <v>62916</v>
       </c>
       <c r="E17" t="s">
         <v>56</v>
       </c>
       <c r="F17" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G17" t="s">
         <v>133</v>
@@ -1869,22 +1881,22 @@
         <v>185</v>
       </c>
       <c r="K17" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L17">
-        <v>699</v>
+        <v>350</v>
       </c>
       <c r="M17">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N17" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="O17" t="s">
         <v>231</v>
       </c>
       <c r="P17">
-        <v>60636</v>
+        <v>76842</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -1892,19 +1904,19 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>100496</v>
+        <v>98465</v>
       </c>
       <c r="C18">
-        <v>241908</v>
-      </c>
-      <c r="D18">
-        <v>39413</v>
+        <v>312044</v>
+      </c>
+      <c r="D18" t="s">
+        <v>25</v>
       </c>
       <c r="E18" t="s">
         <v>57</v>
       </c>
       <c r="F18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G18" t="s">
         <v>134</v>
@@ -1919,22 +1931,22 @@
         <v>185</v>
       </c>
       <c r="K18" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L18">
-        <v>699</v>
+        <v>499</v>
       </c>
       <c r="M18">
         <v>11</v>
       </c>
       <c r="N18" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="O18" t="s">
         <v>231</v>
       </c>
       <c r="P18">
-        <v>54257</v>
+        <v>76811</v>
       </c>
     </row>
     <row r="19" spans="1:16">
@@ -1942,19 +1954,19 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>100503</v>
+        <v>100487</v>
       </c>
       <c r="C19">
-        <v>360991</v>
-      </c>
-      <c r="D19" t="s">
-        <v>30</v>
+        <v>48666</v>
+      </c>
+      <c r="D19">
+        <v>46524</v>
       </c>
       <c r="E19" t="s">
         <v>58</v>
       </c>
       <c r="F19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G19" t="s">
         <v>135</v>
@@ -1969,16 +1981,19 @@
         <v>185</v>
       </c>
       <c r="K19" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L19">
-        <v>649</v>
-      </c>
-      <c r="M19" t="s">
-        <v>191</v>
+        <v>549</v>
+      </c>
+      <c r="M19">
+        <v>11</v>
+      </c>
+      <c r="N19" t="s">
+        <v>203</v>
       </c>
       <c r="O19" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="20" spans="1:16">
@@ -1986,25 +2001,25 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>100521</v>
+        <v>99047</v>
       </c>
       <c r="C20">
-        <v>266562</v>
+        <v>38715</v>
       </c>
       <c r="D20">
-        <v>64066</v>
+        <v>36587</v>
       </c>
       <c r="E20" t="s">
         <v>59</v>
       </c>
       <c r="F20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G20" t="s">
         <v>136</v>
       </c>
       <c r="H20" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I20">
         <v>0</v>
@@ -2016,16 +2031,16 @@
         <v>187</v>
       </c>
       <c r="L20">
-        <v>499</v>
-      </c>
-      <c r="M20">
-        <v>11</v>
-      </c>
-      <c r="N20" t="s">
-        <v>204</v>
+        <v>399</v>
+      </c>
+      <c r="M20" t="s">
+        <v>191</v>
       </c>
       <c r="O20" t="s">
-        <v>231</v>
+        <v>230</v>
+      </c>
+      <c r="P20">
+        <v>57290</v>
       </c>
     </row>
     <row r="21" spans="1:16">
@@ -2033,19 +2048,19 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>99056</v>
+        <v>100494</v>
       </c>
       <c r="C21">
-        <v>76774</v>
+        <v>346010</v>
       </c>
       <c r="D21">
-        <v>74576</v>
+        <v>88175</v>
       </c>
       <c r="E21" t="s">
         <v>60</v>
       </c>
       <c r="F21" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="G21" t="s">
         <v>137</v>
@@ -2063,16 +2078,16 @@
         <v>188</v>
       </c>
       <c r="L21">
-        <v>399</v>
-      </c>
-      <c r="M21" t="s">
-        <v>191</v>
+        <v>999</v>
+      </c>
+      <c r="M21">
+        <v>11</v>
+      </c>
+      <c r="N21" t="s">
+        <v>204</v>
       </c>
       <c r="O21" t="s">
-        <v>230</v>
-      </c>
-      <c r="P21">
-        <v>24188</v>
+        <v>231</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -2080,25 +2095,25 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>99889</v>
+        <v>100501</v>
       </c>
       <c r="C22">
-        <v>17586</v>
+        <v>347090</v>
       </c>
       <c r="D22">
-        <v>16499</v>
+        <v>89255</v>
       </c>
       <c r="E22" t="s">
         <v>61</v>
       </c>
       <c r="F22" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="G22" t="s">
         <v>138</v>
       </c>
       <c r="H22" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="I22">
         <v>0</v>
@@ -2110,7 +2125,7 @@
         <v>188</v>
       </c>
       <c r="L22">
-        <v>499</v>
+        <v>549</v>
       </c>
       <c r="M22">
         <v>11</v>
@@ -2120,9 +2135,6 @@
       </c>
       <c r="O22" t="s">
         <v>231</v>
-      </c>
-      <c r="P22">
-        <v>95586</v>
       </c>
     </row>
     <row r="23" spans="1:16">
@@ -2130,25 +2142,25 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>98466</v>
+        <v>100512</v>
       </c>
       <c r="C23">
-        <v>205081</v>
-      </c>
-      <c r="D23" t="s">
-        <v>31</v>
+        <v>140437</v>
+      </c>
+      <c r="D23">
+        <v>38064</v>
       </c>
       <c r="E23" t="s">
         <v>62</v>
       </c>
       <c r="F23" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="G23" t="s">
         <v>139</v>
       </c>
       <c r="H23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="I23">
         <v>0</v>
@@ -2157,13 +2169,13 @@
         <v>185</v>
       </c>
       <c r="K23" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L23">
-        <v>499</v>
+        <v>449</v>
       </c>
       <c r="M23">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N23" t="s">
         <v>206</v>
@@ -2172,7 +2184,7 @@
         <v>231</v>
       </c>
       <c r="P23">
-        <v>76809</v>
+        <v>55808</v>
       </c>
     </row>
     <row r="24" spans="1:16">
@@ -2180,25 +2192,25 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>98517</v>
+        <v>99332</v>
       </c>
       <c r="C24">
-        <v>232630</v>
+        <v>257916</v>
       </c>
       <c r="D24">
-        <v>30135</v>
+        <v>55420</v>
       </c>
       <c r="E24" t="s">
         <v>63</v>
       </c>
       <c r="F24" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G24" t="s">
         <v>140</v>
       </c>
       <c r="H24" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I24">
         <v>0</v>
@@ -2207,22 +2219,19 @@
         <v>185</v>
       </c>
       <c r="K24" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L24">
-        <v>449</v>
-      </c>
-      <c r="M24">
-        <v>5</v>
-      </c>
-      <c r="N24" t="s">
-        <v>207</v>
+        <v>399</v>
+      </c>
+      <c r="M24" t="s">
+        <v>191</v>
       </c>
       <c r="O24" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="P24">
-        <v>49260</v>
+        <v>73999</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -2230,13 +2239,13 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>98583</v>
+        <v>100493</v>
       </c>
       <c r="C25">
-        <v>114721</v>
-      </c>
-      <c r="D25">
-        <v>12446</v>
+        <v>360045</v>
+      </c>
+      <c r="D25" t="s">
+        <v>26</v>
       </c>
       <c r="E25" t="s">
         <v>64</v>
@@ -2260,16 +2269,13 @@
         <v>188</v>
       </c>
       <c r="L25">
-        <v>399</v>
+        <v>799</v>
       </c>
       <c r="M25" t="s">
         <v>191</v>
       </c>
       <c r="O25" t="s">
         <v>230</v>
-      </c>
-      <c r="P25">
-        <v>11835</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -2277,19 +2283,19 @@
         <v>24</v>
       </c>
       <c r="B26">
-        <v>100489</v>
+        <v>100495</v>
       </c>
       <c r="C26">
-        <v>360888</v>
-      </c>
-      <c r="D26" t="s">
-        <v>32</v>
+        <v>349026</v>
+      </c>
+      <c r="D26">
+        <v>91191</v>
       </c>
       <c r="E26" t="s">
         <v>65</v>
       </c>
       <c r="F26" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="G26" t="s">
         <v>142</v>
@@ -2304,16 +2310,19 @@
         <v>185</v>
       </c>
       <c r="K26" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L26">
         <v>649</v>
       </c>
-      <c r="M26" t="s">
-        <v>191</v>
+      <c r="M26">
+        <v>11</v>
+      </c>
+      <c r="N26" t="s">
+        <v>207</v>
       </c>
       <c r="O26" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -2321,13 +2330,13 @@
         <v>25</v>
       </c>
       <c r="B27">
-        <v>100491</v>
+        <v>100502</v>
       </c>
       <c r="C27">
-        <v>56971</v>
-      </c>
-      <c r="D27">
-        <v>54822</v>
+        <v>205459</v>
+      </c>
+      <c r="D27" t="s">
+        <v>27</v>
       </c>
       <c r="E27" t="s">
         <v>66</v>
@@ -2348,13 +2357,13 @@
         <v>185</v>
       </c>
       <c r="K27" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L27">
-        <v>449</v>
+        <v>399</v>
       </c>
       <c r="M27">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N27" t="s">
         <v>208</v>
@@ -2363,7 +2372,7 @@
         <v>231</v>
       </c>
       <c r="P27">
-        <v>68495</v>
+        <v>38806</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -2371,19 +2380,19 @@
         <v>26</v>
       </c>
       <c r="B28">
-        <v>100508</v>
+        <v>100504</v>
       </c>
       <c r="C28">
-        <v>361018</v>
+        <v>361003</v>
       </c>
       <c r="D28" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E28" t="s">
         <v>67</v>
       </c>
       <c r="F28" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="G28" t="s">
         <v>144</v>
@@ -2398,7 +2407,7 @@
         <v>185</v>
       </c>
       <c r="K28" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L28">
         <v>649</v>
@@ -2415,25 +2424,25 @@
         <v>27</v>
       </c>
       <c r="B29">
-        <v>100523</v>
+        <v>98541</v>
       </c>
       <c r="C29">
-        <v>177956</v>
+        <v>25207</v>
       </c>
       <c r="D29">
-        <v>75463</v>
+        <v>23149</v>
       </c>
       <c r="E29" t="s">
         <v>68</v>
       </c>
       <c r="F29" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G29" t="s">
         <v>145</v>
       </c>
       <c r="H29" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I29">
         <v>0</v>
@@ -2442,13 +2451,13 @@
         <v>185</v>
       </c>
       <c r="K29" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L29">
-        <v>499</v>
+        <v>449</v>
       </c>
       <c r="M29">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N29" t="s">
         <v>209</v>
@@ -2457,7 +2466,7 @@
         <v>231</v>
       </c>
       <c r="P29">
-        <v>4701</v>
+        <v>49403</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -2465,25 +2474,25 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>99840</v>
+        <v>98810</v>
       </c>
       <c r="C30">
-        <v>178067</v>
+        <v>59822</v>
       </c>
       <c r="D30">
-        <v>75574</v>
+        <v>57663</v>
       </c>
       <c r="E30" t="s">
         <v>69</v>
       </c>
       <c r="F30" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G30" t="s">
         <v>146</v>
       </c>
       <c r="H30" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I30">
         <v>0</v>
@@ -2492,19 +2501,22 @@
         <v>185</v>
       </c>
       <c r="K30" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L30">
-        <v>449</v>
-      </c>
-      <c r="M30" t="s">
-        <v>191</v>
+        <v>399</v>
+      </c>
+      <c r="M30">
+        <v>11</v>
+      </c>
+      <c r="N30" t="s">
+        <v>210</v>
       </c>
       <c r="O30" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="P30">
-        <v>74406</v>
+        <v>8024</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -2512,25 +2524,25 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>95940</v>
+        <v>99846</v>
       </c>
       <c r="C31">
-        <v>95151</v>
+        <v>253406</v>
       </c>
       <c r="D31">
-        <v>92910</v>
+        <v>50910</v>
       </c>
       <c r="E31" t="s">
         <v>70</v>
       </c>
       <c r="F31" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="G31" t="s">
         <v>147</v>
       </c>
       <c r="H31" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="I31">
         <v>0</v>
@@ -2539,7 +2551,7 @@
         <v>185</v>
       </c>
       <c r="K31" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L31">
         <v>499</v>
@@ -2548,13 +2560,13 @@
         <v>11</v>
       </c>
       <c r="N31" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="O31" t="s">
         <v>231</v>
       </c>
       <c r="P31">
-        <v>52003</v>
+        <v>79273</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -2562,25 +2574,25 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>100177</v>
+        <v>97773</v>
       </c>
       <c r="C32">
-        <v>194060</v>
+        <v>348244</v>
       </c>
       <c r="D32">
-        <v>91567</v>
+        <v>90409</v>
       </c>
       <c r="E32" t="s">
         <v>71</v>
       </c>
       <c r="F32" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G32" t="s">
         <v>148</v>
       </c>
       <c r="H32" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="I32">
         <v>0</v>
@@ -2589,19 +2601,22 @@
         <v>185</v>
       </c>
       <c r="K32" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L32">
-        <v>499</v>
-      </c>
-      <c r="M32" t="s">
-        <v>191</v>
+        <v>549</v>
+      </c>
+      <c r="M32">
+        <v>11</v>
+      </c>
+      <c r="N32" t="s">
+        <v>212</v>
       </c>
       <c r="O32" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="P32">
-        <v>4813</v>
+        <v>97756</v>
       </c>
     </row>
     <row r="33" spans="1:16">
@@ -2609,19 +2624,19 @@
         <v>31</v>
       </c>
       <c r="B33">
-        <v>100443</v>
+        <v>100331</v>
       </c>
       <c r="C33">
-        <v>354766</v>
+        <v>22791</v>
       </c>
       <c r="D33">
-        <v>96930</v>
+        <v>21685</v>
       </c>
       <c r="E33" t="s">
         <v>72</v>
       </c>
       <c r="F33" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G33" t="s">
         <v>149</v>
@@ -2639,16 +2654,16 @@
         <v>187</v>
       </c>
       <c r="L33">
-        <v>549</v>
-      </c>
-      <c r="M33">
-        <v>11</v>
-      </c>
-      <c r="N33" t="s">
-        <v>211</v>
+        <v>399</v>
+      </c>
+      <c r="M33" t="s">
+        <v>191</v>
       </c>
       <c r="O33" t="s">
-        <v>231</v>
+        <v>230</v>
+      </c>
+      <c r="P33">
+        <v>79141</v>
       </c>
     </row>
     <row r="34" spans="1:16">
@@ -2656,19 +2671,19 @@
         <v>32</v>
       </c>
       <c r="B34">
-        <v>100484</v>
+        <v>100499</v>
       </c>
       <c r="C34">
-        <v>42885</v>
+        <v>79792</v>
       </c>
       <c r="D34">
-        <v>40755</v>
+        <v>77591</v>
       </c>
       <c r="E34" t="s">
         <v>73</v>
       </c>
       <c r="F34" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="G34" t="s">
         <v>150</v>
@@ -2683,16 +2698,19 @@
         <v>185</v>
       </c>
       <c r="K34" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L34">
-        <v>649</v>
-      </c>
-      <c r="M34" t="s">
-        <v>191</v>
+        <v>549</v>
+      </c>
+      <c r="M34">
+        <v>11</v>
+      </c>
+      <c r="N34" t="s">
+        <v>213</v>
       </c>
       <c r="O34" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="35" spans="1:16">
@@ -2700,25 +2718,25 @@
         <v>33</v>
       </c>
       <c r="B35">
-        <v>100486</v>
+        <v>100514</v>
       </c>
       <c r="C35">
-        <v>360869</v>
+        <v>361054</v>
       </c>
       <c r="D35" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E35" t="s">
         <v>74</v>
       </c>
       <c r="F35" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="G35" t="s">
         <v>151</v>
       </c>
       <c r="H35" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I35">
         <v>0</v>
@@ -2727,16 +2745,19 @@
         <v>185</v>
       </c>
       <c r="K35" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L35">
         <v>649</v>
       </c>
-      <c r="M35" t="s">
-        <v>191</v>
+      <c r="M35">
+        <v>11</v>
+      </c>
+      <c r="N35" t="s">
+        <v>214</v>
       </c>
       <c r="O35" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="36" spans="1:16">
@@ -2744,19 +2765,19 @@
         <v>34</v>
       </c>
       <c r="B36">
-        <v>100509</v>
+        <v>97892</v>
       </c>
       <c r="C36">
-        <v>141351</v>
+        <v>151685</v>
       </c>
       <c r="D36">
-        <v>38969</v>
+        <v>49250</v>
       </c>
       <c r="E36" t="s">
         <v>75</v>
       </c>
       <c r="F36" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G36" t="s">
         <v>152</v>
@@ -2771,22 +2792,22 @@
         <v>185</v>
       </c>
       <c r="K36" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L36">
-        <v>699</v>
+        <v>399</v>
       </c>
       <c r="M36">
         <v>11</v>
       </c>
       <c r="N36" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="O36" t="s">
         <v>231</v>
       </c>
       <c r="P36">
-        <v>76258</v>
+        <v>2308</v>
       </c>
     </row>
     <row r="37" spans="1:16">
@@ -2794,25 +2815,25 @@
         <v>35</v>
       </c>
       <c r="B37">
-        <v>100511</v>
+        <v>99890</v>
       </c>
       <c r="C37">
-        <v>361026</v>
-      </c>
-      <c r="D37" t="s">
-        <v>35</v>
+        <v>34927</v>
+      </c>
+      <c r="D37">
+        <v>32841</v>
       </c>
       <c r="E37" t="s">
         <v>76</v>
       </c>
       <c r="F37" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="G37" t="s">
         <v>153</v>
       </c>
       <c r="H37" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I37">
         <v>0</v>
@@ -2824,13 +2845,19 @@
         <v>187</v>
       </c>
       <c r="L37">
-        <v>649</v>
-      </c>
-      <c r="M37" t="s">
-        <v>191</v>
+        <v>499</v>
+      </c>
+      <c r="M37">
+        <v>11</v>
+      </c>
+      <c r="N37" t="s">
+        <v>216</v>
       </c>
       <c r="O37" t="s">
-        <v>230</v>
+        <v>231</v>
+      </c>
+      <c r="P37">
+        <v>95584</v>
       </c>
     </row>
     <row r="38" spans="1:16">
@@ -2838,19 +2865,19 @@
         <v>36</v>
       </c>
       <c r="B38">
-        <v>99080</v>
+        <v>98369</v>
       </c>
       <c r="C38">
-        <v>326105</v>
+        <v>56575</v>
       </c>
       <c r="D38">
-        <v>23044</v>
+        <v>54426</v>
       </c>
       <c r="E38" t="s">
         <v>77</v>
       </c>
       <c r="F38" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G38" t="s">
         <v>154</v>
@@ -2865,19 +2892,22 @@
         <v>185</v>
       </c>
       <c r="K38" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L38">
-        <v>599</v>
-      </c>
-      <c r="M38" t="s">
-        <v>191</v>
+        <v>499</v>
+      </c>
+      <c r="M38">
+        <v>11</v>
+      </c>
+      <c r="N38" t="s">
+        <v>217</v>
       </c>
       <c r="O38" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="P38">
-        <v>83122</v>
+        <v>91270</v>
       </c>
     </row>
     <row r="39" spans="1:16">
@@ -2885,13 +2915,13 @@
         <v>37</v>
       </c>
       <c r="B39">
-        <v>100331</v>
+        <v>100107</v>
       </c>
       <c r="C39">
-        <v>22791</v>
-      </c>
-      <c r="D39">
-        <v>21685</v>
+        <v>312465</v>
+      </c>
+      <c r="D39" t="s">
+        <v>30</v>
       </c>
       <c r="E39" t="s">
         <v>78</v>
@@ -2903,7 +2933,7 @@
         <v>155</v>
       </c>
       <c r="H39" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I39">
         <v>0</v>
@@ -2912,19 +2942,22 @@
         <v>185</v>
       </c>
       <c r="K39" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L39">
-        <v>399</v>
-      </c>
-      <c r="M39" t="s">
-        <v>191</v>
+        <v>549</v>
+      </c>
+      <c r="M39">
+        <v>5</v>
+      </c>
+      <c r="N39" t="s">
+        <v>218</v>
       </c>
       <c r="O39" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="P39">
-        <v>79141</v>
+        <v>77036</v>
       </c>
     </row>
     <row r="40" spans="1:16">
@@ -2932,25 +2965,25 @@
         <v>38</v>
       </c>
       <c r="B40">
-        <v>97773</v>
+        <v>100488</v>
       </c>
       <c r="C40">
-        <v>348244</v>
-      </c>
-      <c r="D40">
-        <v>90409</v>
+        <v>360887</v>
+      </c>
+      <c r="D40" t="s">
+        <v>31</v>
       </c>
       <c r="E40" t="s">
         <v>79</v>
       </c>
       <c r="F40" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="G40" t="s">
         <v>156</v>
       </c>
       <c r="H40" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="I40">
         <v>0</v>
@@ -2968,13 +3001,10 @@
         <v>11</v>
       </c>
       <c r="N40" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="O40" t="s">
         <v>231</v>
-      </c>
-      <c r="P40">
-        <v>97756</v>
       </c>
     </row>
     <row r="41" spans="1:16">
@@ -2982,19 +3012,19 @@
         <v>39</v>
       </c>
       <c r="B41">
-        <v>97892</v>
+        <v>100490</v>
       </c>
       <c r="C41">
-        <v>151685</v>
-      </c>
-      <c r="D41">
-        <v>49250</v>
+        <v>360892</v>
+      </c>
+      <c r="D41" t="s">
+        <v>32</v>
       </c>
       <c r="E41" t="s">
         <v>80</v>
       </c>
       <c r="F41" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="G41" t="s">
         <v>157</v>
@@ -3012,19 +3042,13 @@
         <v>188</v>
       </c>
       <c r="L41">
-        <v>399</v>
-      </c>
-      <c r="M41">
-        <v>11</v>
-      </c>
-      <c r="N41" t="s">
-        <v>214</v>
+        <v>649</v>
+      </c>
+      <c r="M41" t="s">
+        <v>191</v>
       </c>
       <c r="O41" t="s">
-        <v>231</v>
-      </c>
-      <c r="P41">
-        <v>2308</v>
+        <v>230</v>
       </c>
     </row>
     <row r="42" spans="1:16">
@@ -3032,19 +3056,19 @@
         <v>40</v>
       </c>
       <c r="B42">
-        <v>100499</v>
+        <v>100492</v>
       </c>
       <c r="C42">
-        <v>79792</v>
-      </c>
-      <c r="D42">
-        <v>77591</v>
+        <v>360904</v>
+      </c>
+      <c r="D42" t="s">
+        <v>33</v>
       </c>
       <c r="E42" t="s">
         <v>81</v>
       </c>
       <c r="F42" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="G42" t="s">
         <v>158</v>
@@ -3059,7 +3083,7 @@
         <v>185</v>
       </c>
       <c r="K42" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L42">
         <v>549</v>
@@ -3068,7 +3092,7 @@
         <v>11</v>
       </c>
       <c r="N42" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="O42" t="s">
         <v>231</v>
@@ -3079,25 +3103,25 @@
         <v>41</v>
       </c>
       <c r="B43">
-        <v>100514</v>
+        <v>100505</v>
       </c>
       <c r="C43">
-        <v>361054</v>
+        <v>360757</v>
       </c>
       <c r="D43" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E43" t="s">
         <v>82</v>
       </c>
       <c r="F43" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="G43" t="s">
         <v>159</v>
       </c>
       <c r="H43" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="I43">
         <v>0</v>
@@ -3106,16 +3130,16 @@
         <v>185</v>
       </c>
       <c r="K43" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L43">
-        <v>649</v>
+        <v>549</v>
       </c>
       <c r="M43">
         <v>11</v>
       </c>
       <c r="N43" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="O43" t="s">
         <v>231</v>
@@ -3126,25 +3150,25 @@
         <v>42</v>
       </c>
       <c r="B44">
-        <v>98541</v>
+        <v>100507</v>
       </c>
       <c r="C44">
-        <v>25207</v>
+        <v>353643</v>
       </c>
       <c r="D44">
-        <v>23149</v>
+        <v>95807</v>
       </c>
       <c r="E44" t="s">
         <v>83</v>
       </c>
       <c r="F44" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G44" t="s">
         <v>160</v>
       </c>
       <c r="H44" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="I44">
         <v>0</v>
@@ -3156,19 +3180,16 @@
         <v>188</v>
       </c>
       <c r="L44">
-        <v>449</v>
+        <v>649</v>
       </c>
       <c r="M44">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="N44" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="O44" t="s">
         <v>231</v>
-      </c>
-      <c r="P44">
-        <v>49403</v>
       </c>
     </row>
     <row r="45" spans="1:16">
@@ -3176,25 +3197,25 @@
         <v>43</v>
       </c>
       <c r="B45">
-        <v>98810</v>
+        <v>100522</v>
       </c>
       <c r="C45">
-        <v>59822</v>
-      </c>
-      <c r="D45">
-        <v>57663</v>
+        <v>360630</v>
+      </c>
+      <c r="D45" t="s">
+        <v>35</v>
       </c>
       <c r="E45" t="s">
         <v>84</v>
       </c>
       <c r="F45" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G45" t="s">
         <v>161</v>
       </c>
       <c r="H45" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I45">
         <v>0</v>
@@ -3206,19 +3227,13 @@
         <v>188</v>
       </c>
       <c r="L45">
-        <v>399</v>
-      </c>
-      <c r="M45">
-        <v>11</v>
-      </c>
-      <c r="N45" t="s">
-        <v>218</v>
+        <v>549</v>
+      </c>
+      <c r="M45" t="s">
+        <v>191</v>
       </c>
       <c r="O45" t="s">
-        <v>231</v>
-      </c>
-      <c r="P45">
-        <v>8024</v>
+        <v>230</v>
       </c>
     </row>
     <row r="46" spans="1:16">
@@ -3226,25 +3241,25 @@
         <v>44</v>
       </c>
       <c r="B46">
-        <v>99846</v>
+        <v>95940</v>
       </c>
       <c r="C46">
-        <v>253406</v>
+        <v>95151</v>
       </c>
       <c r="D46">
-        <v>50910</v>
+        <v>92910</v>
       </c>
       <c r="E46" t="s">
         <v>85</v>
       </c>
       <c r="F46" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="G46" t="s">
         <v>162</v>
       </c>
       <c r="H46" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="I46">
         <v>0</v>
@@ -3253,7 +3268,7 @@
         <v>185</v>
       </c>
       <c r="K46" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L46">
         <v>499</v>
@@ -3262,13 +3277,13 @@
         <v>11</v>
       </c>
       <c r="N46" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="O46" t="s">
         <v>231</v>
       </c>
       <c r="P46">
-        <v>79273</v>
+        <v>52003</v>
       </c>
     </row>
     <row r="47" spans="1:16">
@@ -3276,19 +3291,19 @@
         <v>45</v>
       </c>
       <c r="B47">
-        <v>100487</v>
+        <v>99080</v>
       </c>
       <c r="C47">
-        <v>48666</v>
+        <v>326105</v>
       </c>
       <c r="D47">
-        <v>46524</v>
+        <v>23044</v>
       </c>
       <c r="E47" t="s">
         <v>86</v>
       </c>
       <c r="F47" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="G47" t="s">
         <v>163</v>
@@ -3306,16 +3321,16 @@
         <v>187</v>
       </c>
       <c r="L47">
-        <v>549</v>
-      </c>
-      <c r="M47">
-        <v>11</v>
-      </c>
-      <c r="N47" t="s">
-        <v>220</v>
+        <v>599</v>
+      </c>
+      <c r="M47" t="s">
+        <v>191</v>
       </c>
       <c r="O47" t="s">
-        <v>231</v>
+        <v>230</v>
+      </c>
+      <c r="P47">
+        <v>83122</v>
       </c>
     </row>
     <row r="48" spans="1:16">
@@ -3323,19 +3338,19 @@
         <v>46</v>
       </c>
       <c r="B48">
-        <v>100494</v>
+        <v>100177</v>
       </c>
       <c r="C48">
-        <v>346010</v>
+        <v>194060</v>
       </c>
       <c r="D48">
-        <v>88175</v>
+        <v>91567</v>
       </c>
       <c r="E48" t="s">
         <v>87</v>
       </c>
       <c r="F48" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G48" t="s">
         <v>164</v>
@@ -3353,16 +3368,16 @@
         <v>187</v>
       </c>
       <c r="L48">
-        <v>999</v>
-      </c>
-      <c r="M48">
-        <v>11</v>
-      </c>
-      <c r="N48" t="s">
-        <v>221</v>
+        <v>499</v>
+      </c>
+      <c r="M48" t="s">
+        <v>191</v>
       </c>
       <c r="O48" t="s">
-        <v>231</v>
+        <v>230</v>
+      </c>
+      <c r="P48">
+        <v>4813</v>
       </c>
     </row>
     <row r="49" spans="1:16">
@@ -3370,19 +3385,19 @@
         <v>47</v>
       </c>
       <c r="B49">
-        <v>100501</v>
+        <v>100443</v>
       </c>
       <c r="C49">
-        <v>347090</v>
+        <v>354766</v>
       </c>
       <c r="D49">
-        <v>89255</v>
+        <v>96930</v>
       </c>
       <c r="E49" t="s">
         <v>88</v>
       </c>
       <c r="F49" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="G49" t="s">
         <v>165</v>
@@ -3397,7 +3412,7 @@
         <v>185</v>
       </c>
       <c r="K49" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L49">
         <v>549</v>
@@ -3406,7 +3421,7 @@
         <v>11</v>
       </c>
       <c r="N49" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="O49" t="s">
         <v>231</v>
@@ -3417,25 +3432,25 @@
         <v>48</v>
       </c>
       <c r="B50">
-        <v>100512</v>
+        <v>100484</v>
       </c>
       <c r="C50">
-        <v>140437</v>
+        <v>42885</v>
       </c>
       <c r="D50">
-        <v>38064</v>
+        <v>40755</v>
       </c>
       <c r="E50" t="s">
         <v>89</v>
       </c>
       <c r="F50" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="G50" t="s">
         <v>166</v>
       </c>
       <c r="H50" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="I50">
         <v>0</v>
@@ -3447,19 +3462,13 @@
         <v>188</v>
       </c>
       <c r="L50">
-        <v>449</v>
-      </c>
-      <c r="M50">
-        <v>5</v>
-      </c>
-      <c r="N50" t="s">
-        <v>223</v>
+        <v>649</v>
+      </c>
+      <c r="M50" t="s">
+        <v>191</v>
       </c>
       <c r="O50" t="s">
-        <v>231</v>
-      </c>
-      <c r="P50">
-        <v>55808</v>
+        <v>230</v>
       </c>
     </row>
     <row r="51" spans="1:16">
@@ -3467,13 +3476,13 @@
         <v>49</v>
       </c>
       <c r="B51">
-        <v>98454</v>
+        <v>100486</v>
       </c>
       <c r="C51">
-        <v>65078</v>
-      </c>
-      <c r="D51">
-        <v>62916</v>
+        <v>360869</v>
+      </c>
+      <c r="D51" t="s">
+        <v>36</v>
       </c>
       <c r="E51" t="s">
         <v>90</v>
@@ -3497,19 +3506,13 @@
         <v>188</v>
       </c>
       <c r="L51">
-        <v>350</v>
-      </c>
-      <c r="M51">
-        <v>5</v>
-      </c>
-      <c r="N51" t="s">
-        <v>224</v>
+        <v>649</v>
+      </c>
+      <c r="M51" t="s">
+        <v>191</v>
       </c>
       <c r="O51" t="s">
-        <v>231</v>
-      </c>
-      <c r="P51">
-        <v>76842</v>
+        <v>230</v>
       </c>
     </row>
     <row r="52" spans="1:16">
@@ -3517,19 +3520,19 @@
         <v>50</v>
       </c>
       <c r="B52">
-        <v>98465</v>
+        <v>100509</v>
       </c>
       <c r="C52">
-        <v>312044</v>
-      </c>
-      <c r="D52" t="s">
-        <v>37</v>
+        <v>141351</v>
+      </c>
+      <c r="D52">
+        <v>38969</v>
       </c>
       <c r="E52" t="s">
         <v>91</v>
       </c>
       <c r="F52" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G52" t="s">
         <v>168</v>
@@ -3544,10 +3547,10 @@
         <v>185</v>
       </c>
       <c r="K52" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L52">
-        <v>499</v>
+        <v>699</v>
       </c>
       <c r="M52">
         <v>11</v>
@@ -3559,7 +3562,7 @@
         <v>231</v>
       </c>
       <c r="P52">
-        <v>76811</v>
+        <v>76258</v>
       </c>
     </row>
     <row r="53" spans="1:16">
@@ -3567,25 +3570,25 @@
         <v>51</v>
       </c>
       <c r="B53">
-        <v>99047</v>
+        <v>100511</v>
       </c>
       <c r="C53">
-        <v>38715</v>
-      </c>
-      <c r="D53">
-        <v>36587</v>
+        <v>361026</v>
+      </c>
+      <c r="D53" t="s">
+        <v>37</v>
       </c>
       <c r="E53" t="s">
         <v>92</v>
       </c>
       <c r="F53" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="G53" t="s">
         <v>169</v>
       </c>
       <c r="H53" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="I53">
         <v>0</v>
@@ -3597,16 +3600,13 @@
         <v>188</v>
       </c>
       <c r="L53">
-        <v>399</v>
+        <v>649</v>
       </c>
       <c r="M53" t="s">
         <v>191</v>
       </c>
       <c r="O53" t="s">
         <v>230</v>
-      </c>
-      <c r="P53">
-        <v>57290</v>
       </c>
     </row>
     <row r="54" spans="1:16">
@@ -3641,7 +3641,7 @@
         <v>185</v>
       </c>
       <c r="K54" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L54">
         <v>1549</v>
@@ -3670,7 +3670,7 @@
         <v>94</v>
       </c>
       <c r="F55" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="G55" t="s">
         <v>171</v>
@@ -3685,7 +3685,7 @@
         <v>185</v>
       </c>
       <c r="K55" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L55">
         <v>649</v>
@@ -3705,25 +3705,25 @@
         <v>54</v>
       </c>
       <c r="B56">
-        <v>100515</v>
+        <v>98943</v>
       </c>
       <c r="C56">
-        <v>361056</v>
-      </c>
-      <c r="D56" t="s">
-        <v>40</v>
+        <v>37106</v>
+      </c>
+      <c r="D56">
+        <v>34985</v>
       </c>
       <c r="E56" t="s">
         <v>95</v>
       </c>
       <c r="F56" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="G56" t="s">
         <v>172</v>
       </c>
       <c r="H56" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="I56">
         <v>0</v>
@@ -3735,16 +3735,16 @@
         <v>187</v>
       </c>
       <c r="L56">
-        <v>649</v>
-      </c>
-      <c r="M56">
-        <v>11</v>
-      </c>
-      <c r="N56" t="s">
-        <v>227</v>
+        <v>399</v>
+      </c>
+      <c r="M56" t="s">
+        <v>191</v>
       </c>
       <c r="O56" t="s">
-        <v>231</v>
+        <v>230</v>
+      </c>
+      <c r="P56">
+        <v>96274</v>
       </c>
     </row>
     <row r="57" spans="1:16">
@@ -3752,25 +3752,25 @@
         <v>55</v>
       </c>
       <c r="B57">
-        <v>98943</v>
+        <v>100515</v>
       </c>
       <c r="C57">
-        <v>37106</v>
-      </c>
-      <c r="D57">
-        <v>34985</v>
+        <v>361056</v>
+      </c>
+      <c r="D57" t="s">
+        <v>40</v>
       </c>
       <c r="E57" t="s">
         <v>96</v>
       </c>
       <c r="F57" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="G57" t="s">
         <v>173</v>
       </c>
       <c r="H57" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I57">
         <v>0</v>
@@ -3782,16 +3782,16 @@
         <v>188</v>
       </c>
       <c r="L57">
-        <v>399</v>
-      </c>
-      <c r="M57" t="s">
-        <v>191</v>
+        <v>649</v>
+      </c>
+      <c r="M57">
+        <v>11</v>
+      </c>
+      <c r="N57" t="s">
+        <v>227</v>
       </c>
       <c r="O57" t="s">
-        <v>230</v>
-      </c>
-      <c r="P57">
-        <v>96274</v>
+        <v>231</v>
       </c>
     </row>
     <row r="58" spans="1:16">
@@ -3811,7 +3811,7 @@
         <v>97</v>
       </c>
       <c r="F58" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="G58" t="s">
         <v>174</v>
@@ -3826,7 +3826,7 @@
         <v>185</v>
       </c>
       <c r="K58" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L58">
         <v>499</v>

</xml_diff>